<commit_message>
CSC: extend to 2070
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\CSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D47818FD-27FB-4FD4-968C-58E44B45BDB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D5B2A59-1A4F-4AEF-8438-CBD6A78A3ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3720" yWindow="3720" windowWidth="43200" windowHeight="17085" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="3" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1076,6 +1076,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1083,7 +1084,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1611,6 +1611,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1618,7 +1619,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2146,6 +2146,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2153,7 +2154,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4274,28 +4274,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3D2DEE-686E-48A0-AC3D-0F54DEA5D0EC}">
   <dimension ref="A1:C124"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="88.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="88.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -4303,40 +4303,40 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A7" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A8" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A11" s="1"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A12" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A14" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -4344,7 +4344,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -4352,7 +4352,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -4360,7 +4360,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -4368,7 +4368,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -4376,7 +4376,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.75">
       <c r="B23">
         <f>(1-EXP(-((C23/$B$19-($B$18-0.5))/$B$16)^$B$17))*$B$15</f>
         <v>0</v>
@@ -4385,7 +4385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.75">
       <c r="B24">
         <f t="shared" ref="B24:B87" si="0">(1-EXP(-((C24/$B$19-($B$18-0.5))/$B$16)^$B$17))*$B$15</f>
         <v>4.0187703366778572E-7</v>
@@ -4394,7 +4394,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.75">
       <c r="B25">
         <f t="shared" si="0"/>
         <v>3.2149861218577768E-6</v>
@@ -4403,7 +4403,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.75">
       <c r="B26">
         <f t="shared" si="0"/>
         <v>1.0850301995346534E-5</v>
@@ -4413,7 +4413,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.75">
       <c r="B27">
         <f t="shared" si="0"/>
         <v>2.571795964551593E-5</v>
@@ -4423,7 +4423,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.75">
       <c r="B28">
         <f t="shared" si="0"/>
         <v>5.0226285691895579E-5</v>
@@ -4433,7 +4433,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.75">
       <c r="B29">
         <f t="shared" si="0"/>
         <v>8.6780443051764905E-5</v>
@@ -4443,7 +4443,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.75">
       <c r="B30">
         <f t="shared" si="0"/>
         <v>1.3778069003070326E-4</v>
@@ -4453,7 +4453,7 @@
         <v>3500</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.75">
       <c r="B31">
         <f t="shared" si="0"/>
         <v>2.0562025564793696E-4</v>
@@ -4463,7 +4463,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.75">
       <c r="B32">
         <f t="shared" si="0"/>
         <v>2.926828338786713E-4</v>
@@ -4473,7 +4473,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B33">
         <f t="shared" si="0"/>
         <v>4.0133970053291554E-4</v>
@@ -4483,7 +4483,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B34">
         <f t="shared" si="0"/>
         <v>5.3394645769462839E-4</v>
@@ -4493,7 +4493,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B35">
         <f t="shared" si="0"/>
         <v>6.9283941201358503E-4</v>
@@ -4503,7 +4503,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B36">
         <f t="shared" si="0"/>
         <v>8.8033159466762703E-4</v>
@@ -4513,7 +4513,7 @@
         <v>6500</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B37">
         <f t="shared" si="0"/>
         <v>1.0987084324921848E-3</v>
@@ -4523,7 +4523,7 @@
         <v>7000</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B38">
         <f t="shared" si="0"/>
         <v>1.3502230815962135E-3</v>
@@ -4533,7 +4533,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B39">
         <f t="shared" si="0"/>
         <v>1.6370914367420941E-3</v>
@@ -4543,7 +4543,7 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B40">
         <f t="shared" si="0"/>
         <v>1.9614868318508726E-3</v>
@@ -4553,7 +4553,7 @@
         <v>8500</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B41">
         <f t="shared" si="0"/>
         <v>2.325534449188732E-3</v>
@@ -4563,7 +4563,7 @@
         <v>9000</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B42">
         <f t="shared" si="0"/>
         <v>2.7313054570853477E-3</v>
@@ -4573,7 +4573,7 @@
         <v>9500</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B43">
         <f t="shared" si="0"/>
         <v>3.1808108984106021E-3</v>
@@ -4583,7 +4583,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B44">
         <f t="shared" si="0"/>
         <v>3.6759953544767184E-3</v>
@@ -4593,7 +4593,7 @@
         <v>10500</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B45">
         <f t="shared" si="0"/>
         <v>4.2187304115184395E-3</v>
@@ -4603,7 +4603,7 @@
         <v>11000</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B46">
         <f t="shared" si="0"/>
         <v>4.8108079594126937E-3</v>
@@ -4613,7 +4613,7 @@
         <v>11500</v>
       </c>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B47">
         <f t="shared" si="0"/>
         <v>5.4539333548070607E-3</v>
@@ -4623,7 +4623,7 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B48">
         <f t="shared" si="0"/>
         <v>6.149718483310862E-3</v>
@@ -4633,7 +4633,7 @@
         <v>12500</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B49">
         <f t="shared" si="0"/>
         <v>6.899674757832674E-3</v>
@@ -4643,7 +4643,7 @@
         <v>13000</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B50">
         <f t="shared" si="0"/>
         <v>7.7052060925004657E-3</v>
@@ -4653,7 +4653,7 @@
         <v>13500</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B51">
         <f t="shared" si="0"/>
         <v>8.5676018938412868E-3</v>
@@ -4663,7 +4663,7 @@
         <v>14000</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B52">
         <f t="shared" si="0"/>
         <v>9.4880301129990352E-3</v>
@@ -4673,7 +4673,7 @@
         <v>14500</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B53">
         <f t="shared" si="0"/>
         <v>1.0467530404697972E-2</v>
@@ -4683,7 +4683,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B54">
         <f t="shared" si="0"/>
         <v>1.1507007440385136E-2</v>
@@ -4693,7 +4693,7 @@
         <v>15500</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B55">
         <f t="shared" si="0"/>
         <v>1.2607224424474078E-2</v>
@@ -4703,7 +4703,7 @@
         <v>16000</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B56">
         <f t="shared" si="0"/>
         <v>1.3768796863832604E-2</v>
@@ -4713,7 +4713,7 @@
         <v>16500</v>
       </c>
     </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B57">
         <f t="shared" si="0"/>
         <v>1.4992186641577837E-2</v>
@@ -4723,7 +4723,7 @@
         <v>17000</v>
       </c>
     </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B58">
         <f t="shared" si="0"/>
         <v>1.6277696446830824E-2</v>
@@ -4733,7 +4733,7 @@
         <v>17500</v>
       </c>
     </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B59">
         <f t="shared" si="0"/>
         <v>1.7625464612310682E-2</v>
@@ -4743,7 +4743,7 @@
         <v>18000</v>
       </c>
     </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B60">
         <f t="shared" si="0"/>
         <v>1.9035460411488268E-2</v>
@@ -4753,7 +4753,7 @@
         <v>18500</v>
       </c>
     </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B61">
         <f t="shared" si="0"/>
         <v>2.0507479866443433E-2</v>
@@ -4763,7 +4763,7 @@
         <v>19000</v>
       </c>
     </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B62">
         <f t="shared" si="0"/>
         <v>2.2041142116558832E-2</v>
@@ -4773,7 +4773,7 @@
         <v>19500</v>
       </c>
     </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B63">
         <f t="shared" si="0"/>
         <v>2.3635886396712456E-2</v>
@@ -4783,7 +4783,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B64">
         <f t="shared" si="0"/>
         <v>2.5290969671690554E-2</v>
@@ -4793,7 +4793,7 @@
         <v>20500</v>
       </c>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B65">
         <f t="shared" si="0"/>
         <v>2.7005464971113717E-2</v>
@@ -4803,7 +4803,7 @@
         <v>21000</v>
       </c>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B66">
         <f t="shared" si="0"/>
         <v>2.8778260466251364E-2</v>
@@ -4813,7 +4813,7 @@
         <v>21500</v>
       </c>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B67">
         <f t="shared" si="0"/>
         <v>3.0608059326685061E-2</v>
@@ -4823,7 +4823,7 @@
         <v>22000</v>
       </c>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B68">
         <f t="shared" si="0"/>
         <v>3.249338039087727E-2</v>
@@ -4833,7 +4833,7 @@
         <v>22500</v>
       </c>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B69">
         <f t="shared" si="0"/>
         <v>3.4432559680315195E-2</v>
@@ -4843,7 +4843,7 @@
         <v>23000</v>
       </c>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B70">
         <f t="shared" si="0"/>
         <v>3.6423752782045189E-2</v>
@@ -4853,7 +4853,7 @@
         <v>23500</v>
       </c>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B71">
         <f t="shared" si="0"/>
         <v>3.8464938119114063E-2</v>
@@ -4863,7 +4863,7 @@
         <v>24000</v>
       </c>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B72">
         <f t="shared" si="0"/>
         <v>4.055392112271447E-2</v>
@@ -4873,7 +4873,7 @@
         <v>24500</v>
       </c>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B73">
         <f t="shared" si="0"/>
         <v>4.2688339313730859E-2</v>
@@ -4883,7 +4883,7 @@
         <v>25000</v>
       </c>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B74">
         <f t="shared" si="0"/>
         <v>4.4865668294935525E-2</v>
@@ -4893,7 +4893,7 @@
         <v>25500</v>
       </c>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B75">
         <f t="shared" si="0"/>
         <v>4.7083228648343023E-2</v>
@@ -4903,7 +4903,7 @@
         <v>26000</v>
       </c>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B76">
         <f t="shared" si="0"/>
         <v>4.9338193725244575E-2</v>
@@ -4913,7 +4913,7 @@
         <v>26500</v>
       </c>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B77">
         <f t="shared" si="0"/>
         <v>5.1627598309274762E-2</v>
@@ -4923,7 +4923,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B78">
         <f t="shared" si="0"/>
         <v>5.3948348125570124E-2</v>
@@ -4933,7 +4933,7 @@
         <v>27500</v>
       </c>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B79">
         <f t="shared" si="0"/>
         <v>5.629723016173821E-2</v>
@@ -4943,7 +4943,7 @@
         <v>28000</v>
       </c>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B80">
         <f t="shared" si="0"/>
         <v>5.8670923759033294E-2</v>
@@ -4953,7 +4953,7 @@
         <v>28500</v>
       </c>
     </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B81">
         <f t="shared" si="0"/>
         <v>6.1066012424913607E-2</v>
@@ -4963,7 +4963,7 @@
         <v>29000</v>
       </c>
     </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B82">
         <f t="shared" si="0"/>
         <v>6.3478996311107899E-2</v>
@@ -4973,7 +4973,7 @@
         <v>29500</v>
       </c>
     </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B83">
         <f t="shared" si="0"/>
         <v>6.5906305294534395E-2</v>
@@ -4983,7 +4983,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B84">
         <f t="shared" si="0"/>
         <v>6.8344312591966452E-2</v>
@@ -4993,7 +4993,7 @@
         <v>30500</v>
       </c>
     </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B85">
         <f t="shared" si="0"/>
         <v>7.0789348833315488E-2</v>
@@ -5003,7 +5003,7 @@
         <v>31000</v>
       </c>
     </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B86">
         <f t="shared" si="0"/>
         <v>7.3237716512875015E-2</v>
@@ -5013,7 +5013,7 @@
         <v>31500</v>
       </c>
     </row>
-    <row r="87" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B87">
         <f t="shared" si="0"/>
         <v>7.5685704732924589E-2</v>
@@ -5023,7 +5023,7 @@
         <v>32000</v>
       </c>
     </row>
-    <row r="88" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B88">
         <f t="shared" ref="B88:B124" si="2">(1-EXP(-((C88/$B$19-($B$18-0.5))/$B$16)^$B$17))*$B$15</f>
         <v>7.8129604149794987E-2</v>
@@ -5033,7 +5033,7 @@
         <v>32500</v>
       </c>
     </row>
-    <row r="89" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B89">
         <f t="shared" si="2"/>
         <v>8.0565722028919276E-2</v>
@@ -5043,7 +5043,7 @@
         <v>33000</v>
       </c>
     </row>
-    <row r="90" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B90">
         <f t="shared" si="2"/>
         <v>8.2990397312597802E-2</v>
@@ -5053,7 +5053,7 @@
         <v>33500</v>
       </c>
     </row>
-    <row r="91" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B91">
         <f t="shared" si="2"/>
         <v>8.5400015602243903E-2</v>
@@ -5063,7 +5063,7 @@
         <v>34000</v>
       </c>
     </row>
-    <row r="92" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B92">
         <f t="shared" si="2"/>
         <v>8.7791023955795813E-2</v>
@@ -5073,7 +5073,7 @@
         <v>34500</v>
       </c>
     </row>
-    <row r="93" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B93">
         <f t="shared" si="2"/>
         <v>9.015994540081855E-2</v>
@@ -5083,7 +5083,7 @@
         <v>35000</v>
       </c>
     </row>
-    <row r="94" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B94">
         <f t="shared" si="2"/>
         <v>9.2503393064599676E-2</v>
@@ -5093,7 +5093,7 @@
         <v>35500</v>
       </c>
     </row>
-    <row r="95" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B95">
         <f t="shared" si="2"/>
         <v>9.4818083824283653E-2</v>
@@ -5103,7 +5103,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="96" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B96">
         <f t="shared" si="2"/>
         <v>9.7100851382792161E-2</v>
@@ -5113,7 +5113,7 @@
         <v>36500</v>
       </c>
     </row>
-    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B97">
         <f t="shared" si="2"/>
         <v>9.9348658679935559E-2</v>
@@ -5123,7 +5123,7 @@
         <v>37000</v>
       </c>
     </row>
-    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B98">
         <f t="shared" si="2"/>
         <v>0.10155860955271043</v>
@@ -5133,7 +5133,7 @@
         <v>37500</v>
       </c>
     </row>
-    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B99">
         <f t="shared" si="2"/>
         <v>0.10372795956427108</v>
@@ -5143,7 +5143,7 @@
         <v>38000</v>
       </c>
     </row>
-    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B100">
         <f t="shared" si="2"/>
         <v>0.10585412592740542</v>
@@ -5153,7 +5153,7 @@
         <v>38500</v>
       </c>
     </row>
-    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B101">
         <f t="shared" si="2"/>
         <v>0.10793469645549059</v>
@@ -5163,7 +5163,7 @@
         <v>39000</v>
       </c>
     </row>
-    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B102">
         <f t="shared" si="2"/>
         <v>0.10996743748177233</v>
@@ -5173,7 +5173,7 @@
         <v>39500</v>
       </c>
     </row>
-    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B103">
         <f t="shared" si="2"/>
         <v>0.11195030069632968</v>
@@ -5183,7 +5183,7 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="104" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B104">
         <f t="shared" si="2"/>
         <v>0.11388142885916275</v>
@@ -5193,7 +5193,7 @@
         <v>40500</v>
       </c>
     </row>
-    <row r="105" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B105">
         <f t="shared" si="2"/>
         <v>0.11575916035737591</v>
@@ -5203,7 +5203,7 @@
         <v>41000</v>
       </c>
     </row>
-    <row r="106" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B106">
         <f t="shared" si="2"/>
         <v>0.11758203258431722</v>
@@ -5213,7 +5213,7 @@
         <v>41500</v>
       </c>
     </row>
-    <row r="107" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B107">
         <f t="shared" si="2"/>
         <v>0.11934878412866376</v>
@@ -5223,7 +5223,7 @@
         <v>42000</v>
       </c>
     </row>
-    <row r="108" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B108">
         <f t="shared" si="2"/>
         <v>0.12105835577169748</v>
@@ -5233,7 +5233,7 @@
         <v>42500</v>
       </c>
     </row>
-    <row r="109" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B109">
         <f t="shared" si="2"/>
         <v>0.12270989030127519</v>
@@ -5243,7 +5243,7 @@
         <v>43000</v>
       </c>
     </row>
-    <row r="110" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B110">
         <f t="shared" si="2"/>
         <v>0.12430273116113988</v>
@@ -5253,7 +5253,7 @@
         <v>43500</v>
       </c>
     </row>
-    <row r="111" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B111">
         <f t="shared" si="2"/>
         <v>0.12583641996413128</v>
@@ -5263,7 +5263,7 @@
         <v>44000</v>
       </c>
     </row>
-    <row r="112" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B112">
         <f t="shared" si="2"/>
         <v>0.12731069290740946</v>
@@ -5273,7 +5273,7 @@
         <v>44500</v>
       </c>
     </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B113">
         <f t="shared" si="2"/>
         <v>0.12872547613689861</v>
@@ -5283,7 +5283,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B114">
         <f t="shared" si="2"/>
         <v>0.1300808801166794</v>
@@ -5293,7 +5293,7 @@
         <v>45500</v>
       </c>
     </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B115">
         <f t="shared" si="2"/>
         <v>0.13137719306690807</v>
@@ -5303,7 +5303,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B116">
         <f t="shared" si="2"/>
         <v>0.13261487354093182</v>
@@ -5313,7 +5313,7 @@
         <v>46500</v>
       </c>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B117">
         <f t="shared" si="2"/>
         <v>0.13379454221852241</v>
@@ -5323,7 +5323,7 @@
         <v>47000</v>
       </c>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B118">
         <f t="shared" si="2"/>
         <v>0.1349169729974935</v>
@@ -5333,7 +5333,7 @@
         <v>47500</v>
       </c>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B119">
         <f t="shared" si="2"/>
         <v>0.1359830834703562</v>
@@ -5343,7 +5343,7 @@
         <v>48000</v>
       </c>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B120">
         <f t="shared" si="2"/>
         <v>0.13699392487605058</v>
@@ -5353,7 +5353,7 @@
         <v>48500</v>
       </c>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B121">
         <f t="shared" si="2"/>
         <v>0.13795067161915198</v>
@@ -5363,7 +5363,7 @@
         <v>49000</v>
       </c>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B122">
         <f t="shared" si="2"/>
         <v>0.13885461045027209</v>
@@ -5373,7 +5373,7 @@
         <v>49500</v>
       </c>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B123">
         <f t="shared" si="2"/>
         <v>0.13970712940166313</v>
@@ -5383,7 +5383,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:3" x14ac:dyDescent="0.75">
       <c r="B124">
         <f t="shared" si="2"/>
         <v>0.14050970657130474</v>
@@ -5405,13 +5405,13 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:CF2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:84" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -5748,7 +5748,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="2" spans="1:84" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:84" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -6095,17 +6095,17 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A2" s="1" t="s">
         <v>34</v>
       </c>
@@ -6123,13 +6123,13 @@
   <sheetPr>
     <tabColor rgb="FF002060"/>
   </sheetPr>
-  <dimension ref="A1:AE25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AZ25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -6223,8 +6223,71 @@
       <c r="AE1">
         <v>2050</v>
       </c>
-    </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF1">
+        <v>2051</v>
+      </c>
+      <c r="AG1">
+        <v>2052</v>
+      </c>
+      <c r="AH1">
+        <v>2053</v>
+      </c>
+      <c r="AI1">
+        <v>2054</v>
+      </c>
+      <c r="AJ1">
+        <v>2055</v>
+      </c>
+      <c r="AK1">
+        <v>2056</v>
+      </c>
+      <c r="AL1">
+        <v>2057</v>
+      </c>
+      <c r="AM1">
+        <v>2058</v>
+      </c>
+      <c r="AN1">
+        <v>2059</v>
+      </c>
+      <c r="AO1">
+        <v>2060</v>
+      </c>
+      <c r="AP1">
+        <v>2061</v>
+      </c>
+      <c r="AQ1">
+        <v>2062</v>
+      </c>
+      <c r="AR1">
+        <v>2063</v>
+      </c>
+      <c r="AS1">
+        <v>2064</v>
+      </c>
+      <c r="AT1">
+        <v>2065</v>
+      </c>
+      <c r="AU1">
+        <v>2066</v>
+      </c>
+      <c r="AV1">
+        <v>2067</v>
+      </c>
+      <c r="AW1">
+        <v>2068</v>
+      </c>
+      <c r="AX1">
+        <v>2069</v>
+      </c>
+      <c r="AY1">
+        <v>2070</v>
+      </c>
+      <c r="AZ1">
+        <v>2071</v>
+      </c>
+    </row>
+    <row r="2" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -6318,8 +6381,71 @@
       <c r="AE2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF2">
+        <v>1</v>
+      </c>
+      <c r="AG2">
+        <v>1</v>
+      </c>
+      <c r="AH2">
+        <v>1</v>
+      </c>
+      <c r="AI2">
+        <v>1</v>
+      </c>
+      <c r="AJ2">
+        <v>1</v>
+      </c>
+      <c r="AK2">
+        <v>1</v>
+      </c>
+      <c r="AL2">
+        <v>1</v>
+      </c>
+      <c r="AM2">
+        <v>1</v>
+      </c>
+      <c r="AN2">
+        <v>1</v>
+      </c>
+      <c r="AO2">
+        <v>1</v>
+      </c>
+      <c r="AP2">
+        <v>1</v>
+      </c>
+      <c r="AQ2">
+        <v>1</v>
+      </c>
+      <c r="AR2">
+        <v>1</v>
+      </c>
+      <c r="AS2">
+        <v>1</v>
+      </c>
+      <c r="AT2">
+        <v>1</v>
+      </c>
+      <c r="AU2">
+        <v>1</v>
+      </c>
+      <c r="AV2">
+        <v>1</v>
+      </c>
+      <c r="AW2">
+        <v>1</v>
+      </c>
+      <c r="AX2">
+        <v>1</v>
+      </c>
+      <c r="AY2">
+        <v>1</v>
+      </c>
+      <c r="AZ2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6413,8 +6539,71 @@
       <c r="AE3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF3">
+        <v>1</v>
+      </c>
+      <c r="AG3">
+        <v>1</v>
+      </c>
+      <c r="AH3">
+        <v>1</v>
+      </c>
+      <c r="AI3">
+        <v>1</v>
+      </c>
+      <c r="AJ3">
+        <v>1</v>
+      </c>
+      <c r="AK3">
+        <v>1</v>
+      </c>
+      <c r="AL3">
+        <v>1</v>
+      </c>
+      <c r="AM3">
+        <v>1</v>
+      </c>
+      <c r="AN3">
+        <v>1</v>
+      </c>
+      <c r="AO3">
+        <v>1</v>
+      </c>
+      <c r="AP3">
+        <v>1</v>
+      </c>
+      <c r="AQ3">
+        <v>1</v>
+      </c>
+      <c r="AR3">
+        <v>1</v>
+      </c>
+      <c r="AS3">
+        <v>1</v>
+      </c>
+      <c r="AT3">
+        <v>1</v>
+      </c>
+      <c r="AU3">
+        <v>1</v>
+      </c>
+      <c r="AV3">
+        <v>1</v>
+      </c>
+      <c r="AW3">
+        <v>1</v>
+      </c>
+      <c r="AX3">
+        <v>1</v>
+      </c>
+      <c r="AY3">
+        <v>1</v>
+      </c>
+      <c r="AZ3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -6508,8 +6697,71 @@
       <c r="AE4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF4">
+        <v>1</v>
+      </c>
+      <c r="AG4">
+        <v>1</v>
+      </c>
+      <c r="AH4">
+        <v>1</v>
+      </c>
+      <c r="AI4">
+        <v>1</v>
+      </c>
+      <c r="AJ4">
+        <v>1</v>
+      </c>
+      <c r="AK4">
+        <v>1</v>
+      </c>
+      <c r="AL4">
+        <v>1</v>
+      </c>
+      <c r="AM4">
+        <v>1</v>
+      </c>
+      <c r="AN4">
+        <v>1</v>
+      </c>
+      <c r="AO4">
+        <v>1</v>
+      </c>
+      <c r="AP4">
+        <v>1</v>
+      </c>
+      <c r="AQ4">
+        <v>1</v>
+      </c>
+      <c r="AR4">
+        <v>1</v>
+      </c>
+      <c r="AS4">
+        <v>1</v>
+      </c>
+      <c r="AT4">
+        <v>1</v>
+      </c>
+      <c r="AU4">
+        <v>1</v>
+      </c>
+      <c r="AV4">
+        <v>1</v>
+      </c>
+      <c r="AW4">
+        <v>1</v>
+      </c>
+      <c r="AX4">
+        <v>1</v>
+      </c>
+      <c r="AY4">
+        <v>1</v>
+      </c>
+      <c r="AZ4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -6603,8 +6855,71 @@
       <c r="AE5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF5">
+        <v>1</v>
+      </c>
+      <c r="AG5">
+        <v>1</v>
+      </c>
+      <c r="AH5">
+        <v>1</v>
+      </c>
+      <c r="AI5">
+        <v>1</v>
+      </c>
+      <c r="AJ5">
+        <v>1</v>
+      </c>
+      <c r="AK5">
+        <v>1</v>
+      </c>
+      <c r="AL5">
+        <v>1</v>
+      </c>
+      <c r="AM5">
+        <v>1</v>
+      </c>
+      <c r="AN5">
+        <v>1</v>
+      </c>
+      <c r="AO5">
+        <v>1</v>
+      </c>
+      <c r="AP5">
+        <v>1</v>
+      </c>
+      <c r="AQ5">
+        <v>1</v>
+      </c>
+      <c r="AR5">
+        <v>1</v>
+      </c>
+      <c r="AS5">
+        <v>1</v>
+      </c>
+      <c r="AT5">
+        <v>1</v>
+      </c>
+      <c r="AU5">
+        <v>1</v>
+      </c>
+      <c r="AV5">
+        <v>1</v>
+      </c>
+      <c r="AW5">
+        <v>1</v>
+      </c>
+      <c r="AX5">
+        <v>1</v>
+      </c>
+      <c r="AY5">
+        <v>1</v>
+      </c>
+      <c r="AZ5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -6698,8 +7013,71 @@
       <c r="AE6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF6">
+        <v>1</v>
+      </c>
+      <c r="AG6">
+        <v>1</v>
+      </c>
+      <c r="AH6">
+        <v>1</v>
+      </c>
+      <c r="AI6">
+        <v>1</v>
+      </c>
+      <c r="AJ6">
+        <v>1</v>
+      </c>
+      <c r="AK6">
+        <v>1</v>
+      </c>
+      <c r="AL6">
+        <v>1</v>
+      </c>
+      <c r="AM6">
+        <v>1</v>
+      </c>
+      <c r="AN6">
+        <v>1</v>
+      </c>
+      <c r="AO6">
+        <v>1</v>
+      </c>
+      <c r="AP6">
+        <v>1</v>
+      </c>
+      <c r="AQ6">
+        <v>1</v>
+      </c>
+      <c r="AR6">
+        <v>1</v>
+      </c>
+      <c r="AS6">
+        <v>1</v>
+      </c>
+      <c r="AT6">
+        <v>1</v>
+      </c>
+      <c r="AU6">
+        <v>1</v>
+      </c>
+      <c r="AV6">
+        <v>1</v>
+      </c>
+      <c r="AW6">
+        <v>1</v>
+      </c>
+      <c r="AX6">
+        <v>1</v>
+      </c>
+      <c r="AY6">
+        <v>1</v>
+      </c>
+      <c r="AZ6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -6793,8 +7171,71 @@
       <c r="AE7">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF7">
+        <v>0.75</v>
+      </c>
+      <c r="AG7">
+        <v>0.75</v>
+      </c>
+      <c r="AH7">
+        <v>0.75</v>
+      </c>
+      <c r="AI7">
+        <v>0.75</v>
+      </c>
+      <c r="AJ7">
+        <v>0.75</v>
+      </c>
+      <c r="AK7">
+        <v>0.75</v>
+      </c>
+      <c r="AL7">
+        <v>0.75</v>
+      </c>
+      <c r="AM7">
+        <v>0.75</v>
+      </c>
+      <c r="AN7">
+        <v>0.75</v>
+      </c>
+      <c r="AO7">
+        <v>0.75</v>
+      </c>
+      <c r="AP7">
+        <v>0.75</v>
+      </c>
+      <c r="AQ7">
+        <v>0.75</v>
+      </c>
+      <c r="AR7">
+        <v>0.75</v>
+      </c>
+      <c r="AS7">
+        <v>0.75</v>
+      </c>
+      <c r="AT7">
+        <v>0.75</v>
+      </c>
+      <c r="AU7">
+        <v>0.75</v>
+      </c>
+      <c r="AV7">
+        <v>0.75</v>
+      </c>
+      <c r="AW7">
+        <v>0.75</v>
+      </c>
+      <c r="AX7">
+        <v>0.75</v>
+      </c>
+      <c r="AY7">
+        <v>0.75</v>
+      </c>
+      <c r="AZ7">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6888,8 +7329,71 @@
       <c r="AE8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF8">
+        <v>1</v>
+      </c>
+      <c r="AG8">
+        <v>1</v>
+      </c>
+      <c r="AH8">
+        <v>1</v>
+      </c>
+      <c r="AI8">
+        <v>1</v>
+      </c>
+      <c r="AJ8">
+        <v>1</v>
+      </c>
+      <c r="AK8">
+        <v>1</v>
+      </c>
+      <c r="AL8">
+        <v>1</v>
+      </c>
+      <c r="AM8">
+        <v>1</v>
+      </c>
+      <c r="AN8">
+        <v>1</v>
+      </c>
+      <c r="AO8">
+        <v>1</v>
+      </c>
+      <c r="AP8">
+        <v>1</v>
+      </c>
+      <c r="AQ8">
+        <v>1</v>
+      </c>
+      <c r="AR8">
+        <v>1</v>
+      </c>
+      <c r="AS8">
+        <v>1</v>
+      </c>
+      <c r="AT8">
+        <v>1</v>
+      </c>
+      <c r="AU8">
+        <v>1</v>
+      </c>
+      <c r="AV8">
+        <v>1</v>
+      </c>
+      <c r="AW8">
+        <v>1</v>
+      </c>
+      <c r="AX8">
+        <v>1</v>
+      </c>
+      <c r="AY8">
+        <v>1</v>
+      </c>
+      <c r="AZ8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -6983,8 +7487,71 @@
       <c r="AE9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF9">
+        <v>1</v>
+      </c>
+      <c r="AG9">
+        <v>1</v>
+      </c>
+      <c r="AH9">
+        <v>1</v>
+      </c>
+      <c r="AI9">
+        <v>1</v>
+      </c>
+      <c r="AJ9">
+        <v>1</v>
+      </c>
+      <c r="AK9">
+        <v>1</v>
+      </c>
+      <c r="AL9">
+        <v>1</v>
+      </c>
+      <c r="AM9">
+        <v>1</v>
+      </c>
+      <c r="AN9">
+        <v>1</v>
+      </c>
+      <c r="AO9">
+        <v>1</v>
+      </c>
+      <c r="AP9">
+        <v>1</v>
+      </c>
+      <c r="AQ9">
+        <v>1</v>
+      </c>
+      <c r="AR9">
+        <v>1</v>
+      </c>
+      <c r="AS9">
+        <v>1</v>
+      </c>
+      <c r="AT9">
+        <v>1</v>
+      </c>
+      <c r="AU9">
+        <v>1</v>
+      </c>
+      <c r="AV9">
+        <v>1</v>
+      </c>
+      <c r="AW9">
+        <v>1</v>
+      </c>
+      <c r="AX9">
+        <v>1</v>
+      </c>
+      <c r="AY9">
+        <v>1</v>
+      </c>
+      <c r="AZ9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -7078,8 +7645,71 @@
       <c r="AE10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF10">
+        <v>1</v>
+      </c>
+      <c r="AG10">
+        <v>1</v>
+      </c>
+      <c r="AH10">
+        <v>1</v>
+      </c>
+      <c r="AI10">
+        <v>1</v>
+      </c>
+      <c r="AJ10">
+        <v>1</v>
+      </c>
+      <c r="AK10">
+        <v>1</v>
+      </c>
+      <c r="AL10">
+        <v>1</v>
+      </c>
+      <c r="AM10">
+        <v>1</v>
+      </c>
+      <c r="AN10">
+        <v>1</v>
+      </c>
+      <c r="AO10">
+        <v>1</v>
+      </c>
+      <c r="AP10">
+        <v>1</v>
+      </c>
+      <c r="AQ10">
+        <v>1</v>
+      </c>
+      <c r="AR10">
+        <v>1</v>
+      </c>
+      <c r="AS10">
+        <v>1</v>
+      </c>
+      <c r="AT10">
+        <v>1</v>
+      </c>
+      <c r="AU10">
+        <v>1</v>
+      </c>
+      <c r="AV10">
+        <v>1</v>
+      </c>
+      <c r="AW10">
+        <v>1</v>
+      </c>
+      <c r="AX10">
+        <v>1</v>
+      </c>
+      <c r="AY10">
+        <v>1</v>
+      </c>
+      <c r="AZ10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -7173,8 +7803,71 @@
       <c r="AE11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF11">
+        <v>1</v>
+      </c>
+      <c r="AG11">
+        <v>1</v>
+      </c>
+      <c r="AH11">
+        <v>1</v>
+      </c>
+      <c r="AI11">
+        <v>1</v>
+      </c>
+      <c r="AJ11">
+        <v>1</v>
+      </c>
+      <c r="AK11">
+        <v>1</v>
+      </c>
+      <c r="AL11">
+        <v>1</v>
+      </c>
+      <c r="AM11">
+        <v>1</v>
+      </c>
+      <c r="AN11">
+        <v>1</v>
+      </c>
+      <c r="AO11">
+        <v>1</v>
+      </c>
+      <c r="AP11">
+        <v>1</v>
+      </c>
+      <c r="AQ11">
+        <v>1</v>
+      </c>
+      <c r="AR11">
+        <v>1</v>
+      </c>
+      <c r="AS11">
+        <v>1</v>
+      </c>
+      <c r="AT11">
+        <v>1</v>
+      </c>
+      <c r="AU11">
+        <v>1</v>
+      </c>
+      <c r="AV11">
+        <v>1</v>
+      </c>
+      <c r="AW11">
+        <v>1</v>
+      </c>
+      <c r="AX11">
+        <v>1</v>
+      </c>
+      <c r="AY11">
+        <v>1</v>
+      </c>
+      <c r="AZ11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -7268,8 +7961,71 @@
       <c r="AE12">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF12">
+        <v>1</v>
+      </c>
+      <c r="AG12">
+        <v>1</v>
+      </c>
+      <c r="AH12">
+        <v>1</v>
+      </c>
+      <c r="AI12">
+        <v>1</v>
+      </c>
+      <c r="AJ12">
+        <v>1</v>
+      </c>
+      <c r="AK12">
+        <v>1</v>
+      </c>
+      <c r="AL12">
+        <v>1</v>
+      </c>
+      <c r="AM12">
+        <v>1</v>
+      </c>
+      <c r="AN12">
+        <v>1</v>
+      </c>
+      <c r="AO12">
+        <v>1</v>
+      </c>
+      <c r="AP12">
+        <v>1</v>
+      </c>
+      <c r="AQ12">
+        <v>1</v>
+      </c>
+      <c r="AR12">
+        <v>1</v>
+      </c>
+      <c r="AS12">
+        <v>1</v>
+      </c>
+      <c r="AT12">
+        <v>1</v>
+      </c>
+      <c r="AU12">
+        <v>1</v>
+      </c>
+      <c r="AV12">
+        <v>1</v>
+      </c>
+      <c r="AW12">
+        <v>1</v>
+      </c>
+      <c r="AX12">
+        <v>1</v>
+      </c>
+      <c r="AY12">
+        <v>1</v>
+      </c>
+      <c r="AZ12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -7363,8 +8119,71 @@
       <c r="AE13">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF13">
+        <v>1</v>
+      </c>
+      <c r="AG13">
+        <v>1</v>
+      </c>
+      <c r="AH13">
+        <v>1</v>
+      </c>
+      <c r="AI13">
+        <v>1</v>
+      </c>
+      <c r="AJ13">
+        <v>1</v>
+      </c>
+      <c r="AK13">
+        <v>1</v>
+      </c>
+      <c r="AL13">
+        <v>1</v>
+      </c>
+      <c r="AM13">
+        <v>1</v>
+      </c>
+      <c r="AN13">
+        <v>1</v>
+      </c>
+      <c r="AO13">
+        <v>1</v>
+      </c>
+      <c r="AP13">
+        <v>1</v>
+      </c>
+      <c r="AQ13">
+        <v>1</v>
+      </c>
+      <c r="AR13">
+        <v>1</v>
+      </c>
+      <c r="AS13">
+        <v>1</v>
+      </c>
+      <c r="AT13">
+        <v>1</v>
+      </c>
+      <c r="AU13">
+        <v>1</v>
+      </c>
+      <c r="AV13">
+        <v>1</v>
+      </c>
+      <c r="AW13">
+        <v>1</v>
+      </c>
+      <c r="AX13">
+        <v>1</v>
+      </c>
+      <c r="AY13">
+        <v>1</v>
+      </c>
+      <c r="AZ13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -7458,8 +8277,71 @@
       <c r="AE14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF14">
+        <v>1</v>
+      </c>
+      <c r="AG14">
+        <v>1</v>
+      </c>
+      <c r="AH14">
+        <v>1</v>
+      </c>
+      <c r="AI14">
+        <v>1</v>
+      </c>
+      <c r="AJ14">
+        <v>1</v>
+      </c>
+      <c r="AK14">
+        <v>1</v>
+      </c>
+      <c r="AL14">
+        <v>1</v>
+      </c>
+      <c r="AM14">
+        <v>1</v>
+      </c>
+      <c r="AN14">
+        <v>1</v>
+      </c>
+      <c r="AO14">
+        <v>1</v>
+      </c>
+      <c r="AP14">
+        <v>1</v>
+      </c>
+      <c r="AQ14">
+        <v>1</v>
+      </c>
+      <c r="AR14">
+        <v>1</v>
+      </c>
+      <c r="AS14">
+        <v>1</v>
+      </c>
+      <c r="AT14">
+        <v>1</v>
+      </c>
+      <c r="AU14">
+        <v>1</v>
+      </c>
+      <c r="AV14">
+        <v>1</v>
+      </c>
+      <c r="AW14">
+        <v>1</v>
+      </c>
+      <c r="AX14">
+        <v>1</v>
+      </c>
+      <c r="AY14">
+        <v>1</v>
+      </c>
+      <c r="AZ14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -7553,8 +8435,71 @@
       <c r="AE15">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF15">
+        <v>1</v>
+      </c>
+      <c r="AG15">
+        <v>1</v>
+      </c>
+      <c r="AH15">
+        <v>1</v>
+      </c>
+      <c r="AI15">
+        <v>1</v>
+      </c>
+      <c r="AJ15">
+        <v>1</v>
+      </c>
+      <c r="AK15">
+        <v>1</v>
+      </c>
+      <c r="AL15">
+        <v>1</v>
+      </c>
+      <c r="AM15">
+        <v>1</v>
+      </c>
+      <c r="AN15">
+        <v>1</v>
+      </c>
+      <c r="AO15">
+        <v>1</v>
+      </c>
+      <c r="AP15">
+        <v>1</v>
+      </c>
+      <c r="AQ15">
+        <v>1</v>
+      </c>
+      <c r="AR15">
+        <v>1</v>
+      </c>
+      <c r="AS15">
+        <v>1</v>
+      </c>
+      <c r="AT15">
+        <v>1</v>
+      </c>
+      <c r="AU15">
+        <v>1</v>
+      </c>
+      <c r="AV15">
+        <v>1</v>
+      </c>
+      <c r="AW15">
+        <v>1</v>
+      </c>
+      <c r="AX15">
+        <v>1</v>
+      </c>
+      <c r="AY15">
+        <v>1</v>
+      </c>
+      <c r="AZ15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -7648,8 +8593,71 @@
       <c r="AE16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF16">
+        <v>1</v>
+      </c>
+      <c r="AG16">
+        <v>1</v>
+      </c>
+      <c r="AH16">
+        <v>1</v>
+      </c>
+      <c r="AI16">
+        <v>1</v>
+      </c>
+      <c r="AJ16">
+        <v>1</v>
+      </c>
+      <c r="AK16">
+        <v>1</v>
+      </c>
+      <c r="AL16">
+        <v>1</v>
+      </c>
+      <c r="AM16">
+        <v>1</v>
+      </c>
+      <c r="AN16">
+        <v>1</v>
+      </c>
+      <c r="AO16">
+        <v>1</v>
+      </c>
+      <c r="AP16">
+        <v>1</v>
+      </c>
+      <c r="AQ16">
+        <v>1</v>
+      </c>
+      <c r="AR16">
+        <v>1</v>
+      </c>
+      <c r="AS16">
+        <v>1</v>
+      </c>
+      <c r="AT16">
+        <v>1</v>
+      </c>
+      <c r="AU16">
+        <v>1</v>
+      </c>
+      <c r="AV16">
+        <v>1</v>
+      </c>
+      <c r="AW16">
+        <v>1</v>
+      </c>
+      <c r="AX16">
+        <v>1</v>
+      </c>
+      <c r="AY16">
+        <v>1</v>
+      </c>
+      <c r="AZ16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -7743,8 +8751,71 @@
       <c r="AE17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF17">
+        <v>1</v>
+      </c>
+      <c r="AG17">
+        <v>1</v>
+      </c>
+      <c r="AH17">
+        <v>1</v>
+      </c>
+      <c r="AI17">
+        <v>1</v>
+      </c>
+      <c r="AJ17">
+        <v>1</v>
+      </c>
+      <c r="AK17">
+        <v>1</v>
+      </c>
+      <c r="AL17">
+        <v>1</v>
+      </c>
+      <c r="AM17">
+        <v>1</v>
+      </c>
+      <c r="AN17">
+        <v>1</v>
+      </c>
+      <c r="AO17">
+        <v>1</v>
+      </c>
+      <c r="AP17">
+        <v>1</v>
+      </c>
+      <c r="AQ17">
+        <v>1</v>
+      </c>
+      <c r="AR17">
+        <v>1</v>
+      </c>
+      <c r="AS17">
+        <v>1</v>
+      </c>
+      <c r="AT17">
+        <v>1</v>
+      </c>
+      <c r="AU17">
+        <v>1</v>
+      </c>
+      <c r="AV17">
+        <v>1</v>
+      </c>
+      <c r="AW17">
+        <v>1</v>
+      </c>
+      <c r="AX17">
+        <v>1</v>
+      </c>
+      <c r="AY17">
+        <v>1</v>
+      </c>
+      <c r="AZ17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -7838,8 +8909,71 @@
       <c r="AE18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF18">
+        <v>1</v>
+      </c>
+      <c r="AG18">
+        <v>1</v>
+      </c>
+      <c r="AH18">
+        <v>1</v>
+      </c>
+      <c r="AI18">
+        <v>1</v>
+      </c>
+      <c r="AJ18">
+        <v>1</v>
+      </c>
+      <c r="AK18">
+        <v>1</v>
+      </c>
+      <c r="AL18">
+        <v>1</v>
+      </c>
+      <c r="AM18">
+        <v>1</v>
+      </c>
+      <c r="AN18">
+        <v>1</v>
+      </c>
+      <c r="AO18">
+        <v>1</v>
+      </c>
+      <c r="AP18">
+        <v>1</v>
+      </c>
+      <c r="AQ18">
+        <v>1</v>
+      </c>
+      <c r="AR18">
+        <v>1</v>
+      </c>
+      <c r="AS18">
+        <v>1</v>
+      </c>
+      <c r="AT18">
+        <v>1</v>
+      </c>
+      <c r="AU18">
+        <v>1</v>
+      </c>
+      <c r="AV18">
+        <v>1</v>
+      </c>
+      <c r="AW18">
+        <v>1</v>
+      </c>
+      <c r="AX18">
+        <v>1</v>
+      </c>
+      <c r="AY18">
+        <v>1</v>
+      </c>
+      <c r="AZ18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -7933,8 +9067,71 @@
       <c r="AE19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF19">
+        <v>1</v>
+      </c>
+      <c r="AG19">
+        <v>1</v>
+      </c>
+      <c r="AH19">
+        <v>1</v>
+      </c>
+      <c r="AI19">
+        <v>1</v>
+      </c>
+      <c r="AJ19">
+        <v>1</v>
+      </c>
+      <c r="AK19">
+        <v>1</v>
+      </c>
+      <c r="AL19">
+        <v>1</v>
+      </c>
+      <c r="AM19">
+        <v>1</v>
+      </c>
+      <c r="AN19">
+        <v>1</v>
+      </c>
+      <c r="AO19">
+        <v>1</v>
+      </c>
+      <c r="AP19">
+        <v>1</v>
+      </c>
+      <c r="AQ19">
+        <v>1</v>
+      </c>
+      <c r="AR19">
+        <v>1</v>
+      </c>
+      <c r="AS19">
+        <v>1</v>
+      </c>
+      <c r="AT19">
+        <v>1</v>
+      </c>
+      <c r="AU19">
+        <v>1</v>
+      </c>
+      <c r="AV19">
+        <v>1</v>
+      </c>
+      <c r="AW19">
+        <v>1</v>
+      </c>
+      <c r="AX19">
+        <v>1</v>
+      </c>
+      <c r="AY19">
+        <v>1</v>
+      </c>
+      <c r="AZ19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -8028,8 +9225,71 @@
       <c r="AE20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF20">
+        <v>1</v>
+      </c>
+      <c r="AG20">
+        <v>1</v>
+      </c>
+      <c r="AH20">
+        <v>1</v>
+      </c>
+      <c r="AI20">
+        <v>1</v>
+      </c>
+      <c r="AJ20">
+        <v>1</v>
+      </c>
+      <c r="AK20">
+        <v>1</v>
+      </c>
+      <c r="AL20">
+        <v>1</v>
+      </c>
+      <c r="AM20">
+        <v>1</v>
+      </c>
+      <c r="AN20">
+        <v>1</v>
+      </c>
+      <c r="AO20">
+        <v>1</v>
+      </c>
+      <c r="AP20">
+        <v>1</v>
+      </c>
+      <c r="AQ20">
+        <v>1</v>
+      </c>
+      <c r="AR20">
+        <v>1</v>
+      </c>
+      <c r="AS20">
+        <v>1</v>
+      </c>
+      <c r="AT20">
+        <v>1</v>
+      </c>
+      <c r="AU20">
+        <v>1</v>
+      </c>
+      <c r="AV20">
+        <v>1</v>
+      </c>
+      <c r="AW20">
+        <v>1</v>
+      </c>
+      <c r="AX20">
+        <v>1</v>
+      </c>
+      <c r="AY20">
+        <v>1</v>
+      </c>
+      <c r="AZ20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -8123,8 +9383,71 @@
       <c r="AE21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF21">
+        <v>1</v>
+      </c>
+      <c r="AG21">
+        <v>1</v>
+      </c>
+      <c r="AH21">
+        <v>1</v>
+      </c>
+      <c r="AI21">
+        <v>1</v>
+      </c>
+      <c r="AJ21">
+        <v>1</v>
+      </c>
+      <c r="AK21">
+        <v>1</v>
+      </c>
+      <c r="AL21">
+        <v>1</v>
+      </c>
+      <c r="AM21">
+        <v>1</v>
+      </c>
+      <c r="AN21">
+        <v>1</v>
+      </c>
+      <c r="AO21">
+        <v>1</v>
+      </c>
+      <c r="AP21">
+        <v>1</v>
+      </c>
+      <c r="AQ21">
+        <v>1</v>
+      </c>
+      <c r="AR21">
+        <v>1</v>
+      </c>
+      <c r="AS21">
+        <v>1</v>
+      </c>
+      <c r="AT21">
+        <v>1</v>
+      </c>
+      <c r="AU21">
+        <v>1</v>
+      </c>
+      <c r="AV21">
+        <v>1</v>
+      </c>
+      <c r="AW21">
+        <v>1</v>
+      </c>
+      <c r="AX21">
+        <v>1</v>
+      </c>
+      <c r="AY21">
+        <v>1</v>
+      </c>
+      <c r="AZ21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -8218,8 +9541,71 @@
       <c r="AE22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF22">
+        <v>1</v>
+      </c>
+      <c r="AG22">
+        <v>1</v>
+      </c>
+      <c r="AH22">
+        <v>1</v>
+      </c>
+      <c r="AI22">
+        <v>1</v>
+      </c>
+      <c r="AJ22">
+        <v>1</v>
+      </c>
+      <c r="AK22">
+        <v>1</v>
+      </c>
+      <c r="AL22">
+        <v>1</v>
+      </c>
+      <c r="AM22">
+        <v>1</v>
+      </c>
+      <c r="AN22">
+        <v>1</v>
+      </c>
+      <c r="AO22">
+        <v>1</v>
+      </c>
+      <c r="AP22">
+        <v>1</v>
+      </c>
+      <c r="AQ22">
+        <v>1</v>
+      </c>
+      <c r="AR22">
+        <v>1</v>
+      </c>
+      <c r="AS22">
+        <v>1</v>
+      </c>
+      <c r="AT22">
+        <v>1</v>
+      </c>
+      <c r="AU22">
+        <v>1</v>
+      </c>
+      <c r="AV22">
+        <v>1</v>
+      </c>
+      <c r="AW22">
+        <v>1</v>
+      </c>
+      <c r="AX22">
+        <v>1</v>
+      </c>
+      <c r="AY22">
+        <v>1</v>
+      </c>
+      <c r="AZ22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -8313,8 +9699,71 @@
       <c r="AE23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF23">
+        <v>1</v>
+      </c>
+      <c r="AG23">
+        <v>1</v>
+      </c>
+      <c r="AH23">
+        <v>1</v>
+      </c>
+      <c r="AI23">
+        <v>1</v>
+      </c>
+      <c r="AJ23">
+        <v>1</v>
+      </c>
+      <c r="AK23">
+        <v>1</v>
+      </c>
+      <c r="AL23">
+        <v>1</v>
+      </c>
+      <c r="AM23">
+        <v>1</v>
+      </c>
+      <c r="AN23">
+        <v>1</v>
+      </c>
+      <c r="AO23">
+        <v>1</v>
+      </c>
+      <c r="AP23">
+        <v>1</v>
+      </c>
+      <c r="AQ23">
+        <v>1</v>
+      </c>
+      <c r="AR23">
+        <v>1</v>
+      </c>
+      <c r="AS23">
+        <v>1</v>
+      </c>
+      <c r="AT23">
+        <v>1</v>
+      </c>
+      <c r="AU23">
+        <v>1</v>
+      </c>
+      <c r="AV23">
+        <v>1</v>
+      </c>
+      <c r="AW23">
+        <v>1</v>
+      </c>
+      <c r="AX23">
+        <v>1</v>
+      </c>
+      <c r="AY23">
+        <v>1</v>
+      </c>
+      <c r="AZ23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -8408,8 +9857,71 @@
       <c r="AE24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF24">
+        <v>1</v>
+      </c>
+      <c r="AG24">
+        <v>1</v>
+      </c>
+      <c r="AH24">
+        <v>1</v>
+      </c>
+      <c r="AI24">
+        <v>1</v>
+      </c>
+      <c r="AJ24">
+        <v>1</v>
+      </c>
+      <c r="AK24">
+        <v>1</v>
+      </c>
+      <c r="AL24">
+        <v>1</v>
+      </c>
+      <c r="AM24">
+        <v>1</v>
+      </c>
+      <c r="AN24">
+        <v>1</v>
+      </c>
+      <c r="AO24">
+        <v>1</v>
+      </c>
+      <c r="AP24">
+        <v>1</v>
+      </c>
+      <c r="AQ24">
+        <v>1</v>
+      </c>
+      <c r="AR24">
+        <v>1</v>
+      </c>
+      <c r="AS24">
+        <v>1</v>
+      </c>
+      <c r="AT24">
+        <v>1</v>
+      </c>
+      <c r="AU24">
+        <v>1</v>
+      </c>
+      <c r="AV24">
+        <v>1</v>
+      </c>
+      <c r="AW24">
+        <v>1</v>
+      </c>
+      <c r="AX24">
+        <v>1</v>
+      </c>
+      <c r="AY24">
+        <v>1</v>
+      </c>
+      <c r="AZ24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:52" x14ac:dyDescent="0.75">
       <c r="A25" t="s">
         <v>28</v>
       </c>
@@ -8501,6 +10013,69 @@
         <v>1</v>
       </c>
       <c r="AE25">
+        <v>1</v>
+      </c>
+      <c r="AF25">
+        <v>1</v>
+      </c>
+      <c r="AG25">
+        <v>1</v>
+      </c>
+      <c r="AH25">
+        <v>1</v>
+      </c>
+      <c r="AI25">
+        <v>1</v>
+      </c>
+      <c r="AJ25">
+        <v>1</v>
+      </c>
+      <c r="AK25">
+        <v>1</v>
+      </c>
+      <c r="AL25">
+        <v>1</v>
+      </c>
+      <c r="AM25">
+        <v>1</v>
+      </c>
+      <c r="AN25">
+        <v>1</v>
+      </c>
+      <c r="AO25">
+        <v>1</v>
+      </c>
+      <c r="AP25">
+        <v>1</v>
+      </c>
+      <c r="AQ25">
+        <v>1</v>
+      </c>
+      <c r="AR25">
+        <v>1</v>
+      </c>
+      <c r="AS25">
+        <v>1</v>
+      </c>
+      <c r="AT25">
+        <v>1</v>
+      </c>
+      <c r="AU25">
+        <v>1</v>
+      </c>
+      <c r="AV25">
+        <v>1</v>
+      </c>
+      <c r="AW25">
+        <v>1</v>
+      </c>
+      <c r="AX25">
+        <v>1</v>
+      </c>
+      <c r="AY25">
+        <v>1</v>
+      </c>
+      <c r="AZ25">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
CSC up max cost
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D5B2A59-1A4F-4AEF-8438-CBD6A78A3ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A95611E0-384B-474B-A7CC-3F6FC5F659B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="3" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -619,307 +619,307 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="101"/>
                 <c:pt idx="0">
-                  <c:v>4.0187703366778572E-7</c:v>
+                  <c:v>5.3583604489038093E-7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.2149861218577768E-6</c:v>
+                  <c:v>4.286648162477036E-6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.0850301995346534E-5</c:v>
+                  <c:v>1.4467069327128713E-5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.571795964551593E-5</c:v>
+                  <c:v>3.4290612860687911E-5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5.0226285691895579E-5</c:v>
+                  <c:v>6.6968380922527435E-5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.6780443051764905E-5</c:v>
+                  <c:v>1.1570725740235322E-4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.3778069003070326E-4</c:v>
+                  <c:v>1.8370758670760434E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.0562025564793696E-4</c:v>
+                  <c:v>2.7416034086391594E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.926828338786713E-4</c:v>
+                  <c:v>3.9024377850489512E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4.0133970053291554E-4</c:v>
+                  <c:v>5.3511960071055413E-4</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>5.3394645769462839E-4</c:v>
+                  <c:v>7.1192861025950462E-4</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>6.9283941201358503E-4</c:v>
+                  <c:v>9.2378588268478008E-4</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>8.8033159466762703E-4</c:v>
+                  <c:v>1.1737754595568363E-3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1.0987084324921848E-3</c:v>
+                  <c:v>1.4649445766562463E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1.3502230815962135E-3</c:v>
+                  <c:v>1.8002974421282847E-3</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1.6370914367420941E-3</c:v>
+                  <c:v>2.1827885823227922E-3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1.9614868318508726E-3</c:v>
+                  <c:v>2.6153157758011638E-3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2.325534449188732E-3</c:v>
+                  <c:v>3.1007125989183093E-3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2.7313054570853477E-3</c:v>
+                  <c:v>3.6417406094471309E-3</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3.1808108984106021E-3</c:v>
+                  <c:v>4.2410811978808027E-3</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3.6759953544767184E-3</c:v>
+                  <c:v>4.9013271393022924E-3</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>4.2187304115184395E-3</c:v>
+                  <c:v>5.6249738820245872E-3</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>4.8108079594126937E-3</c:v>
+                  <c:v>6.4144106125502594E-3</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>5.4539333548070607E-3</c:v>
+                  <c:v>7.2719111397427484E-3</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>6.149718483310862E-3</c:v>
+                  <c:v>8.1996246444144827E-3</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>6.899674757832674E-3</c:v>
+                  <c:v>9.1995663437769003E-3</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>7.7052060925004657E-3</c:v>
+                  <c:v>1.0273608123333956E-2</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>8.5676018938412868E-3</c:v>
+                  <c:v>1.1423469191788382E-2</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>9.4880301129990352E-3</c:v>
+                  <c:v>1.2650706817332047E-2</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1.0467530404697972E-2</c:v>
+                  <c:v>1.3956707206263963E-2</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>1.1507007440385136E-2</c:v>
+                  <c:v>1.5342676587180182E-2</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>1.2607224424474078E-2</c:v>
+                  <c:v>1.6809632565965439E-2</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>1.3768796863832604E-2</c:v>
+                  <c:v>1.8358395818443476E-2</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>1.4992186641577837E-2</c:v>
+                  <c:v>1.9989582188770449E-2</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>1.6277696446830824E-2</c:v>
+                  <c:v>2.1703595262441103E-2</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>1.7625464612310682E-2</c:v>
+                  <c:v>2.3500619483080909E-2</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>1.9035460411488268E-2</c:v>
+                  <c:v>2.538061388198436E-2</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>2.0507479866443433E-2</c:v>
+                  <c:v>2.7343306488591249E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>2.2041142116558832E-2</c:v>
+                  <c:v>2.9388189488745109E-2</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>2.3635886396712456E-2</c:v>
+                  <c:v>3.1514515195616613E-2</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>2.5290969671690554E-2</c:v>
+                  <c:v>3.372129289558741E-2</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>2.7005464971113717E-2</c:v>
+                  <c:v>3.6007286628151627E-2</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>2.8778260466251364E-2</c:v>
+                  <c:v>3.8371013955001823E-2</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>3.0608059326685061E-2</c:v>
+                  <c:v>4.0810745768913415E-2</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>3.249338039087727E-2</c:v>
+                  <c:v>4.3324507187836363E-2</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>3.4432559680315195E-2</c:v>
+                  <c:v>4.5910079573753593E-2</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>3.6423752782045189E-2</c:v>
+                  <c:v>4.8565003709393588E-2</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>3.8464938119114063E-2</c:v>
+                  <c:v>5.1286584158818753E-2</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>4.055392112271447E-2</c:v>
+                  <c:v>5.407189483028596E-2</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>4.2688339313730859E-2</c:v>
+                  <c:v>5.6917785751641151E-2</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>4.4865668294935525E-2</c:v>
+                  <c:v>5.982089105991404E-2</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>4.7083228648343023E-2</c:v>
+                  <c:v>6.2777638197790697E-2</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>4.9338193725244575E-2</c:v>
+                  <c:v>6.5784258300326109E-2</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>5.1627598309274762E-2</c:v>
+                  <c:v>6.8836797745699688E-2</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>5.3948348125570124E-2</c:v>
+                  <c:v>7.1931130834093512E-2</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>5.629723016173821E-2</c:v>
+                  <c:v>7.506297354898428E-2</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>5.8670923759033294E-2</c:v>
+                  <c:v>7.8227898345377744E-2</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>6.1066012424913607E-2</c:v>
+                  <c:v>8.142134989988481E-2</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>6.3478996311107899E-2</c:v>
+                  <c:v>8.4638661748143884E-2</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>6.5906305294534395E-2</c:v>
+                  <c:v>8.787507372604586E-2</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>6.8344312591966452E-2</c:v>
+                  <c:v>9.1125750122621946E-2</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>7.0789348833315488E-2</c:v>
+                  <c:v>9.438579844442066E-2</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>7.3237716512875015E-2</c:v>
+                  <c:v>9.7650288683833367E-2</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>7.5685704732924589E-2</c:v>
+                  <c:v>0.10091427297723279</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>7.8129604149794987E-2</c:v>
+                  <c:v>0.10417280553305999</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>8.0565722028919276E-2</c:v>
+                  <c:v>0.10742096270522571</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>8.2990397312597802E-2</c:v>
+                  <c:v>0.11065386308346375</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>8.5400015602243903E-2</c:v>
+                  <c:v>0.11386668746965854</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>8.7791023955795813E-2</c:v>
+                  <c:v>0.11705469860772776</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>9.015994540081855E-2</c:v>
+                  <c:v>0.12021326053442474</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>9.2503393064599676E-2</c:v>
+                  <c:v>0.12333785741946623</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>9.4818083824283653E-2</c:v>
+                  <c:v>0.12642411176571153</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>9.7100851382792161E-2</c:v>
+                  <c:v>0.12946780184372289</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>9.9348658679935559E-2</c:v>
+                  <c:v>0.1324648782399141</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>0.10155860955271043</c:v>
+                  <c:v>0.13541147940361392</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>0.10372795956427108</c:v>
+                  <c:v>0.1383039460856948</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>0.10585412592740542</c:v>
+                  <c:v>0.14113883456987392</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>0.10793469645549059</c:v>
+                  <c:v>0.1439129286073208</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>0.10996743748177233</c:v>
+                  <c:v>0.14662324997569645</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>0.11195030069632968</c:v>
+                  <c:v>0.14926706759510625</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>0.11388142885916275</c:v>
+                  <c:v>0.15184190514555035</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>0.11575916035737591</c:v>
+                  <c:v>0.15434554714316789</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>0.11758203258431722</c:v>
+                  <c:v>0.15677604344575632</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>0.11934878412866376</c:v>
+                  <c:v>0.1591317121715517</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>0.12105835577169748</c:v>
+                  <c:v>0.16141114102892998</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>0.12270989030127519</c:v>
+                  <c:v>0.16361318706836692</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>0.12430273116113988</c:v>
+                  <c:v>0.16573697488151984</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>0.12583641996413128</c:v>
+                  <c:v>0.16778189328550838</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>0.12731069290740946</c:v>
+                  <c:v>0.16974759054321262</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>0.12872547613689861</c:v>
+                  <c:v>0.17163396818253152</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>0.1300808801166794</c:v>
+                  <c:v>0.17344117348890589</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>0.13137719306690807</c:v>
+                  <c:v>0.17516959075587743</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>0.13261487354093182</c:v>
+                  <c:v>0.17681983138790913</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>0.13379454221852241</c:v>
+                  <c:v>0.17839272295802988</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>0.1349169729974935</c:v>
+                  <c:v>0.17988929732999137</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>0.1359830834703562</c:v>
+                  <c:v>0.18131077796047496</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>0.13699392487605058</c:v>
+                  <c:v>0.18265856650140078</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>0.13795067161915198</c:v>
+                  <c:v>0.18393422882553601</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>0.13885461045027209</c:v>
+                  <c:v>0.18513948060036278</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>0.13970712940166313</c:v>
+                  <c:v>0.18627617253555084</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>0.14050970657130474</c:v>
+                  <c:v>0.18734627542840634</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1337,124 +1337,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.3563306734076795E-6</c:v>
+                  <c:v>1.8084408978769062E-6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.0850301995346534E-5</c:v>
+                  <c:v>1.4467069327128713E-5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.6616623765417522E-5</c:v>
+                  <c:v>4.8822165020556696E-5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.6780443051764905E-5</c:v>
+                  <c:v>1.1570725740235322E-4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.6944632170386997E-4</c:v>
+                  <c:v>2.2592842893849331E-4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.926828338786713E-4</c:v>
+                  <c:v>3.9024377850489512E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.6450282648525794E-4</c:v>
+                  <c:v>6.1933710198034406E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6.9283941201358503E-4</c:v>
+                  <c:v>9.2378588268478008E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>9.8551779614576844E-4</c:v>
+                  <c:v>1.314023728194358E-3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.3502230815962135E-3</c:v>
+                  <c:v>1.8002974421282847E-3</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.7944642344303095E-3</c:v>
+                  <c:v>2.3926189792404132E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.325534449188732E-3</c:v>
+                  <c:v>3.1007125989183093E-3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.9504682038741957E-3</c:v>
+                  <c:v>3.9339576051655948E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.6759953544767184E-3</c:v>
+                  <c:v>4.9013271393022924E-3</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>4.5084926802983977E-3</c:v>
+                  <c:v>6.0113235737311978E-3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>5.4539333548070607E-3</c:v>
+                  <c:v>7.2719111397427484E-3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>6.5178348808602399E-3</c:v>
+                  <c:v>8.6904465078136549E-3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>7.7052060925004657E-3</c:v>
+                  <c:v>1.0273608123333956E-2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>9.0204938865930274E-3</c:v>
+                  <c:v>1.2027325182124038E-2</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1.0467530404697972E-2</c:v>
+                  <c:v>1.3956707206263963E-2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1.2049481436979681E-2</c:v>
+                  <c:v>1.6065975249306242E-2</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1.3768796863832604E-2</c:v>
+                  <c:v>1.8358395818443476E-2</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1.5627163985386609E-2</c:v>
+                  <c:v>2.0836218647182148E-2</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1.7625464612310682E-2</c:v>
+                  <c:v>2.3500619483080909E-2</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1.9763736801589746E-2</c:v>
+                  <c:v>2.6351649068786332E-2</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>2.2041142116558832E-2</c:v>
+                  <c:v>2.9388189488745109E-2</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>2.4455939269979066E-2</c:v>
+                  <c:v>3.2607919026638753E-2</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>2.7005464971113717E-2</c:v>
+                  <c:v>3.6007286628151627E-2</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>2.9686122741700537E-2</c:v>
+                  <c:v>3.9581496988934053E-2</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>3.249338039087727E-2</c:v>
+                  <c:v>4.3324507187836363E-2</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>3.5421776745385977E-2</c:v>
+                  <c:v>4.7229035660514646E-2</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>3.8464938119114063E-2</c:v>
+                  <c:v>5.1286584158818753E-2</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>4.1615604876098174E-2</c:v>
+                  <c:v>5.5487473168130901E-2</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>4.4865668294935525E-2</c:v>
+                  <c:v>5.982089105991404E-2</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>4.820621778208041E-2</c:v>
+                  <c:v>6.4274957042773889E-2</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>5.1627598309274762E-2</c:v>
+                  <c:v>6.8836797745699688E-2</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>5.5119477769415316E-2</c:v>
+                  <c:v>7.3492637025887084E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>5.8670923759033294E-2</c:v>
+                  <c:v>7.8227898345377744E-2</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>6.2270489108216164E-2</c:v>
+                  <c:v>8.3027318810954889E-2</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>6.5906305294534395E-2</c:v>
+                  <c:v>8.787507372604586E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1463,541 +1463,6 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-5E3E-4506-B7FF-2865DFAAB582}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="1627802751"/>
-        <c:axId val="1627803711"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="1627802751"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1627803711"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="1627803711"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1627802751"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:scatterChart>
-        <c:scatterStyle val="smoothMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>'CSC-CSCCCMvSoECBtY'!$B$2:$AP$2</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="41"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>750</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1500</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2250</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>3000</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>3750</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>4500</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>5250</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>6000</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>6750</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>7500</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>8250</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>9000</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>9750</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>10500</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>11250</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>12000</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>12750</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>13500</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>14250</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>15000</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>15750</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>16500</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>17250</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>18000</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>18750</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>19500</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>20250</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>21000</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>21750</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>22500</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>23250</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>24000</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>24750</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>25500</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>26250</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>27000</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>27750</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>28500</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>29250</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>30000</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>'CSC-CSCCCMvSoECBtY'!$B$1:$AP$1</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="41"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1.3563306734076795E-6</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.0850301995346534E-5</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3.6616623765417522E-5</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>8.6780443051764905E-5</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1.6944632170386997E-4</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2.926828338786713E-4</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>4.6450282648525794E-4</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>6.9283941201358503E-4</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>9.8551779614576844E-4</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1.3502230815962135E-3</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>1.7944642344303095E-3</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>2.325534449188732E-3</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>2.9504682038741957E-3</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>3.6759953544767184E-3</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>4.5084926802983977E-3</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>5.4539333548070607E-3</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>6.5178348808602399E-3</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>7.7052060925004657E-3</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>9.0204938865930274E-3</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>1.0467530404697972E-2</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>1.2049481436979681E-2</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>1.3768796863832604E-2</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>1.5627163985386609E-2</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>1.7625464612310682E-2</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>1.9763736801589746E-2</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>2.2041142116558832E-2</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>2.4455939269979066E-2</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>2.7005464971113717E-2</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>2.9686122741700537E-2</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>3.249338039087727E-2</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>3.5421776745385977E-2</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>3.8464938119114063E-2</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>4.1615604876098174E-2</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>4.4865668294935525E-2</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>4.820621778208041E-2</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>5.1627598309274762E-2</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>5.5119477769415316E-2</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>5.8670923759033294E-2</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>6.2270489108216164E-2</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>6.5906305294534395E-2</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D9CD-43DB-BDE0-8A392742F499}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2229,46 +1694,6 @@
 </file>
 
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -3340,522 +2765,6 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -3927,47 +2836,6 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>100012</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>495300</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>176212</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{19E926C4-5B99-77EC-1DCF-F92850905973}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4274,28 +3142,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3D2DEE-686E-48A0-AC3D-0F54DEA5D0EC}">
   <dimension ref="A1:C124"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="88.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="88.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -4303,48 +3171,48 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>37</v>
       </c>
       <c r="B15">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.75">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -4352,7 +3220,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -4360,7 +3228,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -4368,7 +3236,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -4376,7 +3244,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B23">
         <f>(1-EXP(-((C23/$B$19-($B$18-0.5))/$B$16)^$B$17))*$B$15</f>
         <v>0</v>
@@ -4385,1008 +3253,1008 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B24">
         <f t="shared" ref="B24:B87" si="0">(1-EXP(-((C24/$B$19-($B$18-0.5))/$B$16)^$B$17))*$B$15</f>
-        <v>4.0187703366778572E-7</v>
+        <v>5.3583604489038093E-7</v>
       </c>
       <c r="C24">
         <v>500</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B25">
         <f t="shared" si="0"/>
-        <v>3.2149861218577768E-6</v>
+        <v>4.286648162477036E-6</v>
       </c>
       <c r="C25">
         <v>1000</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B26">
         <f t="shared" si="0"/>
-        <v>1.0850301995346534E-5</v>
+        <v>1.4467069327128713E-5</v>
       </c>
       <c r="C26">
         <f>C25+500</f>
         <v>1500</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B27">
         <f t="shared" si="0"/>
-        <v>2.571795964551593E-5</v>
+        <v>3.4290612860687911E-5</v>
       </c>
       <c r="C27">
         <f t="shared" ref="C27:C90" si="1">C26+500</f>
         <v>2000</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B28">
         <f t="shared" si="0"/>
-        <v>5.0226285691895579E-5</v>
+        <v>6.6968380922527435E-5</v>
       </c>
       <c r="C28">
         <f t="shared" si="1"/>
         <v>2500</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B29">
         <f t="shared" si="0"/>
-        <v>8.6780443051764905E-5</v>
+        <v>1.1570725740235322E-4</v>
       </c>
       <c r="C29">
         <f t="shared" si="1"/>
         <v>3000</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B30">
         <f t="shared" si="0"/>
-        <v>1.3778069003070326E-4</v>
+        <v>1.8370758670760434E-4</v>
       </c>
       <c r="C30">
         <f t="shared" si="1"/>
         <v>3500</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B31">
         <f t="shared" si="0"/>
-        <v>2.0562025564793696E-4</v>
+        <v>2.7416034086391594E-4</v>
       </c>
       <c r="C31">
         <f t="shared" si="1"/>
         <v>4000</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B32">
         <f t="shared" si="0"/>
-        <v>2.926828338786713E-4</v>
+        <v>3.9024377850489512E-4</v>
       </c>
       <c r="C32">
         <f t="shared" si="1"/>
         <v>4500</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33">
         <f t="shared" si="0"/>
-        <v>4.0133970053291554E-4</v>
+        <v>5.3511960071055413E-4</v>
       </c>
       <c r="C33">
         <f t="shared" si="1"/>
         <v>5000</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34">
         <f t="shared" si="0"/>
-        <v>5.3394645769462839E-4</v>
+        <v>7.1192861025950462E-4</v>
       </c>
       <c r="C34">
         <f t="shared" si="1"/>
         <v>5500</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35">
         <f t="shared" si="0"/>
-        <v>6.9283941201358503E-4</v>
+        <v>9.2378588268478008E-4</v>
       </c>
       <c r="C35">
         <f t="shared" si="1"/>
         <v>6000</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36">
         <f t="shared" si="0"/>
-        <v>8.8033159466762703E-4</v>
+        <v>1.1737754595568363E-3</v>
       </c>
       <c r="C36">
         <f t="shared" si="1"/>
         <v>6500</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37">
         <f t="shared" si="0"/>
-        <v>1.0987084324921848E-3</v>
+        <v>1.4649445766562463E-3</v>
       </c>
       <c r="C37">
         <f t="shared" si="1"/>
         <v>7000</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38">
         <f t="shared" si="0"/>
-        <v>1.3502230815962135E-3</v>
+        <v>1.8002974421282847E-3</v>
       </c>
       <c r="C38">
         <f t="shared" si="1"/>
         <v>7500</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39">
         <f t="shared" si="0"/>
-        <v>1.6370914367420941E-3</v>
+        <v>2.1827885823227922E-3</v>
       </c>
       <c r="C39">
         <f t="shared" si="1"/>
         <v>8000</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40">
         <f t="shared" si="0"/>
-        <v>1.9614868318508726E-3</v>
+        <v>2.6153157758011638E-3</v>
       </c>
       <c r="C40">
         <f t="shared" si="1"/>
         <v>8500</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41">
         <f t="shared" si="0"/>
-        <v>2.325534449188732E-3</v>
+        <v>3.1007125989183093E-3</v>
       </c>
       <c r="C41">
         <f t="shared" si="1"/>
         <v>9000</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42">
         <f t="shared" si="0"/>
-        <v>2.7313054570853477E-3</v>
+        <v>3.6417406094471309E-3</v>
       </c>
       <c r="C42">
         <f t="shared" si="1"/>
         <v>9500</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43">
         <f t="shared" si="0"/>
-        <v>3.1808108984106021E-3</v>
+        <v>4.2410811978808027E-3</v>
       </c>
       <c r="C43">
         <f t="shared" si="1"/>
         <v>10000</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44">
         <f t="shared" si="0"/>
-        <v>3.6759953544767184E-3</v>
+        <v>4.9013271393022924E-3</v>
       </c>
       <c r="C44">
         <f t="shared" si="1"/>
         <v>10500</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B45">
         <f t="shared" si="0"/>
-        <v>4.2187304115184395E-3</v>
+        <v>5.6249738820245872E-3</v>
       </c>
       <c r="C45">
         <f t="shared" si="1"/>
         <v>11000</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46">
         <f t="shared" si="0"/>
-        <v>4.8108079594126937E-3</v>
+        <v>6.4144106125502594E-3</v>
       </c>
       <c r="C46">
         <f t="shared" si="1"/>
         <v>11500</v>
       </c>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47">
         <f t="shared" si="0"/>
-        <v>5.4539333548070607E-3</v>
+        <v>7.2719111397427484E-3</v>
       </c>
       <c r="C47">
         <f t="shared" si="1"/>
         <v>12000</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48">
         <f t="shared" si="0"/>
-        <v>6.149718483310862E-3</v>
+        <v>8.1996246444144827E-3</v>
       </c>
       <c r="C48">
         <f t="shared" si="1"/>
         <v>12500</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49">
         <f t="shared" si="0"/>
-        <v>6.899674757832674E-3</v>
+        <v>9.1995663437769003E-3</v>
       </c>
       <c r="C49">
         <f t="shared" si="1"/>
         <v>13000</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50">
         <f t="shared" si="0"/>
-        <v>7.7052060925004657E-3</v>
+        <v>1.0273608123333956E-2</v>
       </c>
       <c r="C50">
         <f t="shared" si="1"/>
         <v>13500</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B51">
         <f t="shared" si="0"/>
-        <v>8.5676018938412868E-3</v>
+        <v>1.1423469191788382E-2</v>
       </c>
       <c r="C51">
         <f t="shared" si="1"/>
         <v>14000</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B52">
         <f t="shared" si="0"/>
-        <v>9.4880301129990352E-3</v>
+        <v>1.2650706817332047E-2</v>
       </c>
       <c r="C52">
         <f t="shared" si="1"/>
         <v>14500</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B53">
         <f t="shared" si="0"/>
-        <v>1.0467530404697972E-2</v>
+        <v>1.3956707206263963E-2</v>
       </c>
       <c r="C53">
         <f t="shared" si="1"/>
         <v>15000</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B54">
         <f t="shared" si="0"/>
-        <v>1.1507007440385136E-2</v>
+        <v>1.5342676587180182E-2</v>
       </c>
       <c r="C54">
         <f t="shared" si="1"/>
         <v>15500</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B55">
         <f t="shared" si="0"/>
-        <v>1.2607224424474078E-2</v>
+        <v>1.6809632565965439E-2</v>
       </c>
       <c r="C55">
         <f t="shared" si="1"/>
         <v>16000</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B56">
         <f t="shared" si="0"/>
-        <v>1.3768796863832604E-2</v>
+        <v>1.8358395818443476E-2</v>
       </c>
       <c r="C56">
         <f t="shared" si="1"/>
         <v>16500</v>
       </c>
     </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B57">
         <f t="shared" si="0"/>
-        <v>1.4992186641577837E-2</v>
+        <v>1.9989582188770449E-2</v>
       </c>
       <c r="C57">
         <f t="shared" si="1"/>
         <v>17000</v>
       </c>
     </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B58">
         <f t="shared" si="0"/>
-        <v>1.6277696446830824E-2</v>
+        <v>2.1703595262441103E-2</v>
       </c>
       <c r="C58">
         <f t="shared" si="1"/>
         <v>17500</v>
       </c>
     </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B59">
         <f t="shared" si="0"/>
-        <v>1.7625464612310682E-2</v>
+        <v>2.3500619483080909E-2</v>
       </c>
       <c r="C59">
         <f t="shared" si="1"/>
         <v>18000</v>
       </c>
     </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B60">
         <f t="shared" si="0"/>
-        <v>1.9035460411488268E-2</v>
+        <v>2.538061388198436E-2</v>
       </c>
       <c r="C60">
         <f t="shared" si="1"/>
         <v>18500</v>
       </c>
     </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B61">
         <f t="shared" si="0"/>
-        <v>2.0507479866443433E-2</v>
+        <v>2.7343306488591249E-2</v>
       </c>
       <c r="C61">
         <f t="shared" si="1"/>
         <v>19000</v>
       </c>
     </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B62">
         <f t="shared" si="0"/>
-        <v>2.2041142116558832E-2</v>
+        <v>2.9388189488745109E-2</v>
       </c>
       <c r="C62">
         <f t="shared" si="1"/>
         <v>19500</v>
       </c>
     </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B63">
         <f t="shared" si="0"/>
-        <v>2.3635886396712456E-2</v>
+        <v>3.1514515195616613E-2</v>
       </c>
       <c r="C63">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
     </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B64">
         <f t="shared" si="0"/>
-        <v>2.5290969671690554E-2</v>
+        <v>3.372129289558741E-2</v>
       </c>
       <c r="C64">
         <f t="shared" si="1"/>
         <v>20500</v>
       </c>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B65">
         <f t="shared" si="0"/>
-        <v>2.7005464971113717E-2</v>
+        <v>3.6007286628151627E-2</v>
       </c>
       <c r="C65">
         <f t="shared" si="1"/>
         <v>21000</v>
       </c>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66">
         <f t="shared" si="0"/>
-        <v>2.8778260466251364E-2</v>
+        <v>3.8371013955001823E-2</v>
       </c>
       <c r="C66">
         <f t="shared" si="1"/>
         <v>21500</v>
       </c>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B67">
         <f t="shared" si="0"/>
-        <v>3.0608059326685061E-2</v>
+        <v>4.0810745768913415E-2</v>
       </c>
       <c r="C67">
         <f t="shared" si="1"/>
         <v>22000</v>
       </c>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B68">
         <f t="shared" si="0"/>
-        <v>3.249338039087727E-2</v>
+        <v>4.3324507187836363E-2</v>
       </c>
       <c r="C68">
         <f t="shared" si="1"/>
         <v>22500</v>
       </c>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B69">
         <f t="shared" si="0"/>
-        <v>3.4432559680315195E-2</v>
+        <v>4.5910079573753593E-2</v>
       </c>
       <c r="C69">
         <f t="shared" si="1"/>
         <v>23000</v>
       </c>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B70">
         <f t="shared" si="0"/>
-        <v>3.6423752782045189E-2</v>
+        <v>4.8565003709393588E-2</v>
       </c>
       <c r="C70">
         <f t="shared" si="1"/>
         <v>23500</v>
       </c>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B71">
         <f t="shared" si="0"/>
-        <v>3.8464938119114063E-2</v>
+        <v>5.1286584158818753E-2</v>
       </c>
       <c r="C71">
         <f t="shared" si="1"/>
         <v>24000</v>
       </c>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B72">
         <f t="shared" si="0"/>
-        <v>4.055392112271447E-2</v>
+        <v>5.407189483028596E-2</v>
       </c>
       <c r="C72">
         <f t="shared" si="1"/>
         <v>24500</v>
       </c>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B73">
         <f t="shared" si="0"/>
-        <v>4.2688339313730859E-2</v>
+        <v>5.6917785751641151E-2</v>
       </c>
       <c r="C73">
         <f t="shared" si="1"/>
         <v>25000</v>
       </c>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B74">
         <f t="shared" si="0"/>
-        <v>4.4865668294935525E-2</v>
+        <v>5.982089105991404E-2</v>
       </c>
       <c r="C74">
         <f t="shared" si="1"/>
         <v>25500</v>
       </c>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B75">
         <f t="shared" si="0"/>
-        <v>4.7083228648343023E-2</v>
+        <v>6.2777638197790697E-2</v>
       </c>
       <c r="C75">
         <f t="shared" si="1"/>
         <v>26000</v>
       </c>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B76">
         <f t="shared" si="0"/>
-        <v>4.9338193725244575E-2</v>
+        <v>6.5784258300326109E-2</v>
       </c>
       <c r="C76">
         <f t="shared" si="1"/>
         <v>26500</v>
       </c>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B77">
         <f t="shared" si="0"/>
-        <v>5.1627598309274762E-2</v>
+        <v>6.8836797745699688E-2</v>
       </c>
       <c r="C77">
         <f t="shared" si="1"/>
         <v>27000</v>
       </c>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B78">
         <f t="shared" si="0"/>
-        <v>5.3948348125570124E-2</v>
+        <v>7.1931130834093512E-2</v>
       </c>
       <c r="C78">
         <f t="shared" si="1"/>
         <v>27500</v>
       </c>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B79">
         <f t="shared" si="0"/>
-        <v>5.629723016173821E-2</v>
+        <v>7.506297354898428E-2</v>
       </c>
       <c r="C79">
         <f t="shared" si="1"/>
         <v>28000</v>
       </c>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B80">
         <f t="shared" si="0"/>
-        <v>5.8670923759033294E-2</v>
+        <v>7.8227898345377744E-2</v>
       </c>
       <c r="C80">
         <f t="shared" si="1"/>
         <v>28500</v>
       </c>
     </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B81">
         <f t="shared" si="0"/>
-        <v>6.1066012424913607E-2</v>
+        <v>8.142134989988481E-2</v>
       </c>
       <c r="C81">
         <f t="shared" si="1"/>
         <v>29000</v>
       </c>
     </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B82">
         <f t="shared" si="0"/>
-        <v>6.3478996311107899E-2</v>
+        <v>8.4638661748143884E-2</v>
       </c>
       <c r="C82">
         <f t="shared" si="1"/>
         <v>29500</v>
       </c>
     </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B83">
         <f t="shared" si="0"/>
-        <v>6.5906305294534395E-2</v>
+        <v>8.787507372604586E-2</v>
       </c>
       <c r="C83">
         <f t="shared" si="1"/>
         <v>30000</v>
       </c>
     </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B84">
         <f t="shared" si="0"/>
-        <v>6.8344312591966452E-2</v>
+        <v>9.1125750122621946E-2</v>
       </c>
       <c r="C84">
         <f t="shared" si="1"/>
         <v>30500</v>
       </c>
     </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B85">
         <f t="shared" si="0"/>
-        <v>7.0789348833315488E-2</v>
+        <v>9.438579844442066E-2</v>
       </c>
       <c r="C85">
         <f t="shared" si="1"/>
         <v>31000</v>
       </c>
     </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B86">
         <f t="shared" si="0"/>
-        <v>7.3237716512875015E-2</v>
+        <v>9.7650288683833367E-2</v>
       </c>
       <c r="C86">
         <f t="shared" si="1"/>
         <v>31500</v>
       </c>
     </row>
-    <row r="87" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="87" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B87">
         <f t="shared" si="0"/>
-        <v>7.5685704732924589E-2</v>
+        <v>0.10091427297723279</v>
       </c>
       <c r="C87">
         <f t="shared" si="1"/>
         <v>32000</v>
       </c>
     </row>
-    <row r="88" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="88" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B88">
         <f t="shared" ref="B88:B124" si="2">(1-EXP(-((C88/$B$19-($B$18-0.5))/$B$16)^$B$17))*$B$15</f>
-        <v>7.8129604149794987E-2</v>
+        <v>0.10417280553305999</v>
       </c>
       <c r="C88">
         <f t="shared" si="1"/>
         <v>32500</v>
       </c>
     </row>
-    <row r="89" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="89" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B89">
         <f t="shared" si="2"/>
-        <v>8.0565722028919276E-2</v>
+        <v>0.10742096270522571</v>
       </c>
       <c r="C89">
         <f t="shared" si="1"/>
         <v>33000</v>
       </c>
     </row>
-    <row r="90" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="90" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B90">
         <f t="shared" si="2"/>
-        <v>8.2990397312597802E-2</v>
+        <v>0.11065386308346375</v>
       </c>
       <c r="C90">
         <f t="shared" si="1"/>
         <v>33500</v>
       </c>
     </row>
-    <row r="91" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="91" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B91">
         <f t="shared" si="2"/>
-        <v>8.5400015602243903E-2</v>
+        <v>0.11386668746965854</v>
       </c>
       <c r="C91">
         <f t="shared" ref="C91:C124" si="3">C90+500</f>
         <v>34000</v>
       </c>
     </row>
-    <row r="92" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="92" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B92">
         <f t="shared" si="2"/>
-        <v>8.7791023955795813E-2</v>
+        <v>0.11705469860772776</v>
       </c>
       <c r="C92">
         <f t="shared" si="3"/>
         <v>34500</v>
       </c>
     </row>
-    <row r="93" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="93" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B93">
         <f t="shared" si="2"/>
-        <v>9.015994540081855E-2</v>
+        <v>0.12021326053442474</v>
       </c>
       <c r="C93">
         <f t="shared" si="3"/>
         <v>35000</v>
       </c>
     </row>
-    <row r="94" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="94" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B94">
         <f t="shared" si="2"/>
-        <v>9.2503393064599676E-2</v>
+        <v>0.12333785741946623</v>
       </c>
       <c r="C94">
         <f t="shared" si="3"/>
         <v>35500</v>
       </c>
     </row>
-    <row r="95" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="95" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B95">
         <f t="shared" si="2"/>
-        <v>9.4818083824283653E-2</v>
+        <v>0.12642411176571153</v>
       </c>
       <c r="C95">
         <f t="shared" si="3"/>
         <v>36000</v>
       </c>
     </row>
-    <row r="96" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="96" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B96">
         <f t="shared" si="2"/>
-        <v>9.7100851382792161E-2</v>
+        <v>0.12946780184372289</v>
       </c>
       <c r="C96">
         <f t="shared" si="3"/>
         <v>36500</v>
       </c>
     </row>
-    <row r="97" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B97">
         <f t="shared" si="2"/>
-        <v>9.9348658679935559E-2</v>
+        <v>0.1324648782399141</v>
       </c>
       <c r="C97">
         <f t="shared" si="3"/>
         <v>37000</v>
       </c>
     </row>
-    <row r="98" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B98">
         <f t="shared" si="2"/>
-        <v>0.10155860955271043</v>
+        <v>0.13541147940361392</v>
       </c>
       <c r="C98">
         <f t="shared" si="3"/>
         <v>37500</v>
       </c>
     </row>
-    <row r="99" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B99">
         <f t="shared" si="2"/>
-        <v>0.10372795956427108</v>
+        <v>0.1383039460856948</v>
       </c>
       <c r="C99">
         <f t="shared" si="3"/>
         <v>38000</v>
       </c>
     </row>
-    <row r="100" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B100">
         <f t="shared" si="2"/>
-        <v>0.10585412592740542</v>
+        <v>0.14113883456987392</v>
       </c>
       <c r="C100">
         <f t="shared" si="3"/>
         <v>38500</v>
       </c>
     </row>
-    <row r="101" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B101">
         <f t="shared" si="2"/>
-        <v>0.10793469645549059</v>
+        <v>0.1439129286073208</v>
       </c>
       <c r="C101">
         <f t="shared" si="3"/>
         <v>39000</v>
       </c>
     </row>
-    <row r="102" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B102">
         <f t="shared" si="2"/>
-        <v>0.10996743748177233</v>
+        <v>0.14662324997569645</v>
       </c>
       <c r="C102">
         <f t="shared" si="3"/>
         <v>39500</v>
       </c>
     </row>
-    <row r="103" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B103">
         <f t="shared" si="2"/>
-        <v>0.11195030069632968</v>
+        <v>0.14926706759510625</v>
       </c>
       <c r="C103">
         <f t="shared" si="3"/>
         <v>40000</v>
       </c>
     </row>
-    <row r="104" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="104" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B104">
         <f t="shared" si="2"/>
-        <v>0.11388142885916275</v>
+        <v>0.15184190514555035</v>
       </c>
       <c r="C104">
         <f t="shared" si="3"/>
         <v>40500</v>
       </c>
     </row>
-    <row r="105" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="105" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B105">
         <f t="shared" si="2"/>
-        <v>0.11575916035737591</v>
+        <v>0.15434554714316789</v>
       </c>
       <c r="C105">
         <f t="shared" si="3"/>
         <v>41000</v>
       </c>
     </row>
-    <row r="106" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="106" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B106">
         <f t="shared" si="2"/>
-        <v>0.11758203258431722</v>
+        <v>0.15677604344575632</v>
       </c>
       <c r="C106">
         <f t="shared" si="3"/>
         <v>41500</v>
       </c>
     </row>
-    <row r="107" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="107" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B107">
         <f t="shared" si="2"/>
-        <v>0.11934878412866376</v>
+        <v>0.1591317121715517</v>
       </c>
       <c r="C107">
         <f t="shared" si="3"/>
         <v>42000</v>
       </c>
     </row>
-    <row r="108" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="108" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B108">
         <f t="shared" si="2"/>
-        <v>0.12105835577169748</v>
+        <v>0.16141114102892998</v>
       </c>
       <c r="C108">
         <f t="shared" si="3"/>
         <v>42500</v>
       </c>
     </row>
-    <row r="109" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="109" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B109">
         <f t="shared" si="2"/>
-        <v>0.12270989030127519</v>
+        <v>0.16361318706836692</v>
       </c>
       <c r="C109">
         <f t="shared" si="3"/>
         <v>43000</v>
       </c>
     </row>
-    <row r="110" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="110" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B110">
         <f t="shared" si="2"/>
-        <v>0.12430273116113988</v>
+        <v>0.16573697488151984</v>
       </c>
       <c r="C110">
         <f t="shared" si="3"/>
         <v>43500</v>
       </c>
     </row>
-    <row r="111" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="111" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B111">
         <f t="shared" si="2"/>
-        <v>0.12583641996413128</v>
+        <v>0.16778189328550838</v>
       </c>
       <c r="C111">
         <f t="shared" si="3"/>
         <v>44000</v>
       </c>
     </row>
-    <row r="112" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="112" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B112">
         <f t="shared" si="2"/>
-        <v>0.12731069290740946</v>
+        <v>0.16974759054321262</v>
       </c>
       <c r="C112">
         <f t="shared" si="3"/>
         <v>44500</v>
       </c>
     </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B113">
         <f t="shared" si="2"/>
-        <v>0.12872547613689861</v>
+        <v>0.17163396818253152</v>
       </c>
       <c r="C113">
         <f t="shared" si="3"/>
         <v>45000</v>
       </c>
     </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B114">
         <f t="shared" si="2"/>
-        <v>0.1300808801166794</v>
+        <v>0.17344117348890589</v>
       </c>
       <c r="C114">
         <f t="shared" si="3"/>
         <v>45500</v>
       </c>
     </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B115">
         <f t="shared" si="2"/>
-        <v>0.13137719306690807</v>
+        <v>0.17516959075587743</v>
       </c>
       <c r="C115">
         <f t="shared" si="3"/>
         <v>46000</v>
       </c>
     </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B116">
         <f t="shared" si="2"/>
-        <v>0.13261487354093182</v>
+        <v>0.17681983138790913</v>
       </c>
       <c r="C116">
         <f t="shared" si="3"/>
         <v>46500</v>
       </c>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B117">
         <f t="shared" si="2"/>
-        <v>0.13379454221852241</v>
+        <v>0.17839272295802988</v>
       </c>
       <c r="C117">
         <f t="shared" si="3"/>
         <v>47000</v>
       </c>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B118">
         <f t="shared" si="2"/>
-        <v>0.1349169729974935</v>
+        <v>0.17988929732999137</v>
       </c>
       <c r="C118">
         <f t="shared" si="3"/>
         <v>47500</v>
       </c>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B119">
         <f t="shared" si="2"/>
-        <v>0.1359830834703562</v>
+        <v>0.18131077796047496</v>
       </c>
       <c r="C119">
         <f t="shared" si="3"/>
         <v>48000</v>
       </c>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B120">
         <f t="shared" si="2"/>
-        <v>0.13699392487605058</v>
+        <v>0.18265856650140078</v>
       </c>
       <c r="C120">
         <f t="shared" si="3"/>
         <v>48500</v>
       </c>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B121">
         <f t="shared" si="2"/>
-        <v>0.13795067161915198</v>
+        <v>0.18393422882553601</v>
       </c>
       <c r="C121">
         <f t="shared" si="3"/>
         <v>49000</v>
       </c>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B122">
         <f t="shared" si="2"/>
-        <v>0.13885461045027209</v>
+        <v>0.18513948060036278</v>
       </c>
       <c r="C122">
         <f t="shared" si="3"/>
         <v>49500</v>
       </c>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B123">
         <f t="shared" si="2"/>
-        <v>0.13970712940166313</v>
+        <v>0.18627617253555084</v>
       </c>
       <c r="C123">
         <f t="shared" si="3"/>
         <v>50000</v>
       </c>
     </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.75">
+    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B124">
         <f t="shared" si="2"/>
-        <v>0.14050970657130474</v>
+        <v>0.18734627542840634</v>
       </c>
       <c r="C124">
         <f t="shared" si="3"/>
@@ -5405,13 +4273,13 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:CF2"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -5421,334 +4289,334 @@
       </c>
       <c r="C1">
         <f>(1-EXP(-((C2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.3563306734076795E-6</v>
+        <v>1.8084408978769062E-6</v>
       </c>
       <c r="D1">
         <f>(1-EXP(-((D2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.0850301995346534E-5</v>
+        <v>1.4467069327128713E-5</v>
       </c>
       <c r="E1">
         <f>(1-EXP(-((E2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.6616623765417522E-5</v>
+        <v>4.8822165020556696E-5</v>
       </c>
       <c r="F1">
         <f>(1-EXP(-((F2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.6780443051764905E-5</v>
+        <v>1.1570725740235322E-4</v>
       </c>
       <c r="G1">
         <f>(1-EXP(-((G2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.6944632170386997E-4</v>
+        <v>2.2592842893849331E-4</v>
       </c>
       <c r="H1">
         <f>(1-EXP(-((H2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.926828338786713E-4</v>
+        <v>3.9024377850489512E-4</v>
       </c>
       <c r="I1">
         <f>(1-EXP(-((I2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.6450282648525794E-4</v>
+        <v>6.1933710198034406E-4</v>
       </c>
       <c r="J1">
         <f>(1-EXP(-((J2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.9283941201358503E-4</v>
+        <v>9.2378588268478008E-4</v>
       </c>
       <c r="K1">
         <f>(1-EXP(-((K2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.8551779614576844E-4</v>
+        <v>1.314023728194358E-3</v>
       </c>
       <c r="L1">
         <f>(1-EXP(-((L2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.3502230815962135E-3</v>
+        <v>1.8002974421282847E-3</v>
       </c>
       <c r="M1">
         <f>(1-EXP(-((M2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.7944642344303095E-3</v>
+        <v>2.3926189792404132E-3</v>
       </c>
       <c r="N1">
         <f>(1-EXP(-((N2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.325534449188732E-3</v>
+        <v>3.1007125989183093E-3</v>
       </c>
       <c r="O1">
         <f>(1-EXP(-((O2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.9504682038741957E-3</v>
+        <v>3.9339576051655948E-3</v>
       </c>
       <c r="P1">
         <f>(1-EXP(-((P2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.6759953544767184E-3</v>
+        <v>4.9013271393022924E-3</v>
       </c>
       <c r="Q1">
         <f>(1-EXP(-((Q2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.5084926802983977E-3</v>
+        <v>6.0113235737311978E-3</v>
       </c>
       <c r="R1">
         <f>(1-EXP(-((R2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.4539333548070607E-3</v>
+        <v>7.2719111397427484E-3</v>
       </c>
       <c r="S1">
         <f>(1-EXP(-((S2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.5178348808602399E-3</v>
+        <v>8.6904465078136549E-3</v>
       </c>
       <c r="T1">
         <f>(1-EXP(-((T2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>7.7052060925004657E-3</v>
+        <v>1.0273608123333956E-2</v>
       </c>
       <c r="U1">
         <f>(1-EXP(-((U2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.0204938865930274E-3</v>
+        <v>1.2027325182124038E-2</v>
       </c>
       <c r="V1">
         <f>(1-EXP(-((V2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.0467530404697972E-2</v>
+        <v>1.3956707206263963E-2</v>
       </c>
       <c r="W1">
         <f>(1-EXP(-((W2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.2049481436979681E-2</v>
+        <v>1.6065975249306242E-2</v>
       </c>
       <c r="X1">
         <f>(1-EXP(-((X2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.3768796863832604E-2</v>
+        <v>1.8358395818443476E-2</v>
       </c>
       <c r="Y1">
         <f>(1-EXP(-((Y2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.5627163985386609E-2</v>
+        <v>2.0836218647182148E-2</v>
       </c>
       <c r="Z1">
         <f>(1-EXP(-((Z2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.7625464612310682E-2</v>
+        <v>2.3500619483080909E-2</v>
       </c>
       <c r="AA1">
         <f>(1-EXP(-((AA2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.9763736801589746E-2</v>
+        <v>2.6351649068786332E-2</v>
       </c>
       <c r="AB1">
         <f>(1-EXP(-((AB2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.2041142116558832E-2</v>
+        <v>2.9388189488745109E-2</v>
       </c>
       <c r="AC1">
         <f>(1-EXP(-((AC2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.4455939269979066E-2</v>
+        <v>3.2607919026638753E-2</v>
       </c>
       <c r="AD1">
         <f>(1-EXP(-((AD2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.7005464971113717E-2</v>
+        <v>3.6007286628151627E-2</v>
       </c>
       <c r="AE1">
         <f>(1-EXP(-((AE2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.9686122741700537E-2</v>
+        <v>3.9581496988934053E-2</v>
       </c>
       <c r="AF1">
         <f>(1-EXP(-((AF2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.249338039087727E-2</v>
+        <v>4.3324507187836363E-2</v>
       </c>
       <c r="AG1">
         <f>(1-EXP(-((AG2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.5421776745385977E-2</v>
+        <v>4.7229035660514646E-2</v>
       </c>
       <c r="AH1">
         <f>(1-EXP(-((AH2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.8464938119114063E-2</v>
+        <v>5.1286584158818753E-2</v>
       </c>
       <c r="AI1">
         <f>(1-EXP(-((AI2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.1615604876098174E-2</v>
+        <v>5.5487473168130901E-2</v>
       </c>
       <c r="AJ1">
         <f>(1-EXP(-((AJ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.4865668294935525E-2</v>
+        <v>5.982089105991404E-2</v>
       </c>
       <c r="AK1">
         <f>(1-EXP(-((AK2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.820621778208041E-2</v>
+        <v>6.4274957042773889E-2</v>
       </c>
       <c r="AL1">
         <f>(1-EXP(-((AL2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.1627598309274762E-2</v>
+        <v>6.8836797745699688E-2</v>
       </c>
       <c r="AM1">
         <f>(1-EXP(-((AM2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.5119477769415316E-2</v>
+        <v>7.3492637025887084E-2</v>
       </c>
       <c r="AN1">
         <f>(1-EXP(-((AN2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.8670923759033294E-2</v>
+        <v>7.8227898345377744E-2</v>
       </c>
       <c r="AO1">
         <f>(1-EXP(-((AO2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.2270489108216164E-2</v>
+        <v>8.3027318810954889E-2</v>
       </c>
       <c r="AP1">
         <f>(1-EXP(-((AP2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.5906305294534395E-2</v>
+        <v>8.787507372604586E-2</v>
       </c>
       <c r="AQ1">
         <f>(1-EXP(-((AQ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.9566182700893778E-2</v>
+        <v>9.2754910267858384E-2</v>
       </c>
       <c r="AR1">
         <f>(1-EXP(-((AR2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>7.3237716512875015E-2</v>
+        <v>9.7650288683833367E-2</v>
       </c>
       <c r="AS1">
         <f>(1-EXP(-((AS2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>7.6908396903694956E-2</v>
+        <v>0.10254452920492661</v>
       </c>
       <c r="AT1">
         <f>(1-EXP(-((AT2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.0565722028919276E-2</v>
+        <v>0.10742096270522571</v>
       </c>
       <c r="AU1">
         <f>(1-EXP(-((AU2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.4197312252647025E-2</v>
+        <v>0.11226308300352937</v>
       </c>
       <c r="AV1">
         <f>(1-EXP(-((AV2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.7791023955795813E-2</v>
+        <v>0.11705469860772776</v>
       </c>
       <c r="AW1">
         <f>(1-EXP(-((AW2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.1335061238442886E-2</v>
+        <v>0.12178008165125719</v>
       </c>
       <c r="AX1">
         <f>(1-EXP(-((AX2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.4818083824283653E-2</v>
+        <v>0.12642411176571153</v>
       </c>
       <c r="AY1">
         <f>(1-EXP(-((AY2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.8229309507649534E-2</v>
+        <v>0.13097241267686607</v>
       </c>
       <c r="AZ1">
         <f>(1-EXP(-((AZ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.10155860955271043</v>
+        <v>0.13541147940361392</v>
       </c>
       <c r="BA1">
         <f>(1-EXP(-((BA2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.10479659555998135</v>
+        <v>0.13972879407997515</v>
       </c>
       <c r="BB1">
         <f>(1-EXP(-((BB2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.10793469645549059</v>
+        <v>0.1439129286073208</v>
       </c>
       <c r="BC1">
         <f>(1-EXP(-((BC2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11096522443033115</v>
+        <v>0.14795363257377489</v>
       </c>
       <c r="BD1">
         <f>(1-EXP(-((BD2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11388142885916275</v>
+        <v>0.15184190514555035</v>
       </c>
       <c r="BE1">
         <f>(1-EXP(-((BE2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11667753745097514</v>
+        <v>0.15557004993463353</v>
       </c>
       <c r="BF1">
         <f>(1-EXP(-((BF2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11934878412866376</v>
+        <v>0.1591317121715517</v>
       </c>
       <c r="BG1">
         <f>(1-EXP(-((BG2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12189142338962897</v>
+        <v>0.16252189785283866</v>
       </c>
       <c r="BH1">
         <f>(1-EXP(-((BH2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12430273116113988</v>
+        <v>0.16573697488151984</v>
       </c>
       <c r="BI1">
         <f>(1-EXP(-((BI2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12658099242476617</v>
+        <v>0.16877465656635493</v>
       </c>
       <c r="BJ1">
         <f>(1-EXP(-((BJ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12872547613689861</v>
+        <v>0.17163396818253152</v>
       </c>
       <c r="BK1">
         <f>(1-EXP(-((BK2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.13073639821054656</v>
+        <v>0.17431519761406211</v>
       </c>
       <c r="BL1">
         <f>(1-EXP(-((BL2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.13261487354093182</v>
+        <v>0.17681983138790913</v>
       </c>
       <c r="BM1">
         <f>(1-EXP(-((BM2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.13436285824823427</v>
+        <v>0.17915047766431236</v>
       </c>
       <c r="BN1">
         <f>(1-EXP(-((BN2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.1359830834703562</v>
+        <v>0.18131077796047496</v>
       </c>
       <c r="BO1">
         <f>(1-EXP(-((BO2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.13747898216292775</v>
+        <v>0.18330530955057037</v>
       </c>
       <c r="BP1">
         <f>(1-EXP(-((BP2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.13885461045027209</v>
+        <v>0.18513948060036278</v>
       </c>
       <c r="BQ1">
         <f>(1-EXP(-((BQ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14011456511819612</v>
+        <v>0.18681942015759484</v>
       </c>
       <c r="BR1">
         <f>(1-EXP(-((BR2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14126389884704021</v>
+        <v>0.18835186512938695</v>
       </c>
       <c r="BS1">
         <f>(1-EXP(-((BS2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.1423080347524181</v>
+        <v>0.18974404633655748</v>
       </c>
       <c r="BT1">
         <f>(1-EXP(-((BT2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14325268173371089</v>
+        <v>0.19100357564494788</v>
       </c>
       <c r="BU1">
         <f>(1-EXP(-((BU2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14410375202992939</v>
+        <v>0.19213833603990588</v>
       </c>
       <c r="BV1">
         <f>(1-EXP(-((BV2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.1448672822532501</v>
+        <v>0.1931563763376668</v>
       </c>
       <c r="BW1">
         <f>(1-EXP(-((BW2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14554935901734684</v>
+        <v>0.19406581202312914</v>
       </c>
       <c r="BX1">
         <f>(1-EXP(-((BX2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14615605010611638</v>
+        <v>0.19487473347482187</v>
       </c>
       <c r="BY1">
         <f>(1-EXP(-((BY2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14669334194440264</v>
+        <v>0.19559112259253686</v>
       </c>
       <c r="BZ1">
         <f>(1-EXP(-((BZ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14716708394183772</v>
+        <v>0.19622277858911699</v>
       </c>
       <c r="CA1">
         <f>(1-EXP(-((CA2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14758294008979489</v>
+        <v>0.19677725345305985</v>
       </c>
       <c r="CB1">
         <f>(1-EXP(-((CB2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.1479463480052261</v>
+        <v>0.1972617973403015</v>
       </c>
       <c r="CC1">
         <f>(1-EXP(-((CC2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14826248543885948</v>
+        <v>0.19768331391847932</v>
       </c>
       <c r="CD1">
         <f>(1-EXP(-((CD2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14853624410321731</v>
+        <v>0.19804832547095644</v>
       </c>
       <c r="CE1">
         <f>(1-EXP(-((CE2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.1487722105317654</v>
+        <v>0.19836294737568722</v>
       </c>
       <c r="CF1">
         <f>(1-EXP(-((CF2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:84" x14ac:dyDescent="0.75">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -6080,12 +4948,12 @@
         <v>60750</v>
       </c>
       <c r="CF2" s="2">
-        <v>1000000</v>
+        <f>10^9</f>
+        <v>1000000000</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6095,17 +4963,17 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>34</v>
       </c>
@@ -6124,12 +4992,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:AZ25"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -6287,7 +5155,7 @@
         <v>2071</v>
       </c>
     </row>
-    <row r="2" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -6445,7 +5313,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6603,7 +5471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -6761,7 +5629,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -6919,7 +5787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -7077,7 +5945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -7235,7 +6103,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="8" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -7393,7 +6261,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -7551,7 +6419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -7709,7 +6577,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -7867,7 +6735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -8025,7 +6893,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -8183,7 +7051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -8341,7 +7209,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -8499,7 +7367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -8657,7 +7525,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="17" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -8815,7 +7683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="18" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -8973,7 +7841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="19" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -9131,7 +7999,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="20" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -9289,7 +8157,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="21" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -9447,7 +8315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="22" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -9605,7 +8473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="23" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -9763,7 +8631,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="24" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -9921,7 +8789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:52" x14ac:dyDescent="0.75">
+    <row r="25" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>28</v>
       </c>

</xml_diff>